<commit_message>
Brandbook styling and real logo
</commit_message>
<xml_diff>
--- a/pecan-plan.xlsx
+++ b/pecan-plan.xlsx
@@ -35,7 +35,7 @@
     <font>
       <b/>
       <sz val="10"/>
-      <color rgb="FFF7DC9F"/>
+      <color rgb="FF862837"/>
       <name val="Arial"/>
     </font>
     <font>
@@ -52,7 +52,7 @@
     <font>
       <b/>
       <sz val="8"/>
-      <color rgb="FFF7DC9F"/>
+      <color rgb="FF862837"/>
       <name val="Arial"/>
     </font>
     <font>
@@ -71,7 +71,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF862837"/>
+        <fgColor rgb="FFF7DC9F"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>

</xml_diff>

<commit_message>
Rename role to founders
</commit_message>
<xml_diff>
--- a/pecan-plan.xlsx
+++ b/pecan-plan.xlsx
@@ -454,7 +454,7 @@
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Заказчик</t>
+          <t xml:space="preserve">Основатели PECÀN</t>
         </is>
       </c>
       <c r="E5" s="3"/>
@@ -525,7 +525,7 @@
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Заказчик</t>
+          <t xml:space="preserve">Основатели PECÀN</t>
         </is>
       </c>
       <c r="F6" s="4">
@@ -664,7 +664,7 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Заказчик</t>
+          <t xml:space="preserve">Основатели PECÀN</t>
         </is>
       </c>
       <c r="E8" s="3"/>
@@ -1015,7 +1015,7 @@
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Заказчик</t>
+          <t xml:space="preserve">Основатели PECÀN</t>
         </is>
       </c>
       <c r="F13" s="4">
@@ -1228,7 +1228,7 @@
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Заказчик</t>
+          <t xml:space="preserve">Основатели PECÀN</t>
         </is>
       </c>
       <c r="E16" s="3"/>
@@ -1443,7 +1443,7 @@
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Заказчик</t>
+          <t xml:space="preserve">Основатели PECÀN</t>
         </is>
       </c>
       <c r="F19" s="4">
@@ -1469,7 +1469,7 @@
       </c>
       <c r="M19" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ищем с нуля. Отбор студий с опытом в кофейнях и пекарнях, сравнение сроков и стоимости, выбор вместе с заказчиком. Авторский надзор включаем в договор сразу.</t>
+          <t xml:space="preserve">Ищем с нуля. Отбор студий с опытом в кофейнях и пекарнях, сравнение сроков и стоимости, выбор вместе с основателями PECÀN. Авторский надзор включаем в договор сразу.</t>
         </is>
       </c>
       <c r="N19" s="8"/>
@@ -1516,7 +1516,7 @@
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Заказчик</t>
+          <t xml:space="preserve">Основатели PECÀN</t>
         </is>
       </c>
       <c r="E20" s="3"/>
@@ -1617,7 +1617,7 @@
       </c>
       <c r="M21" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Референсы от заказчика, стилистика по брендбуку, технологическое зонирование от Gastro Ultima.</t>
+          <t xml:space="preserve">Референсы от основателей PECÀN, стилистика по брендбуку, технологическое зонирование от Gastro Ultima.</t>
         </is>
       </c>
       <c r="N21" s="8"/>
@@ -1952,7 +1952,7 @@
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Заказчик</t>
+          <t xml:space="preserve">Основатели PECÀN</t>
         </is>
       </c>
       <c r="E26" s="3" t="inlineStr">
@@ -2101,7 +2101,7 @@
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Заказчик, Gastro Ultima</t>
+          <t xml:space="preserve">Основатели PECÀN, Gastro Ultima</t>
         </is>
       </c>
       <c r="F28" s="4">
@@ -2175,7 +2175,7 @@
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Заказчик</t>
+          <t xml:space="preserve">Основатели PECÀN</t>
         </is>
       </c>
       <c r="F29" s="4">
@@ -2253,7 +2253,7 @@
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Заказчик</t>
+          <t xml:space="preserve">Основатели PECÀN</t>
         </is>
       </c>
       <c r="F30" s="4">
@@ -2326,7 +2326,7 @@
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Заказчик</t>
+          <t xml:space="preserve">Основатели PECÀN</t>
         </is>
       </c>
       <c r="E31" s="3" t="inlineStr">
@@ -2883,7 +2883,7 @@
       </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Заказчик, строители</t>
+          <t xml:space="preserve">Основатели PECÀN, строители</t>
         </is>
       </c>
       <c r="F39" s="4">
@@ -3097,7 +3097,7 @@
       </c>
       <c r="E42" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Заказчик</t>
+          <t xml:space="preserve">Основатели PECÀN</t>
         </is>
       </c>
       <c r="F42" s="4">
@@ -3240,7 +3240,7 @@
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Заказчик</t>
+          <t xml:space="preserve">Основатели PECÀN</t>
         </is>
       </c>
       <c r="E44" s="3"/>
@@ -3319,7 +3319,7 @@
       </c>
       <c r="E45" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Заказчик</t>
+          <t xml:space="preserve">Основатели PECÀN</t>
         </is>
       </c>
       <c r="F45" s="4">
@@ -3392,7 +3392,7 @@
       </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Заказчик</t>
+          <t xml:space="preserve">Основатели PECÀN</t>
         </is>
       </c>
       <c r="E46" s="3" t="inlineStr">
@@ -3466,7 +3466,7 @@
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Заказчик</t>
+          <t xml:space="preserve">Основатели PECÀN</t>
         </is>
       </c>
       <c r="E47" s="3" t="inlineStr">
@@ -4035,7 +4035,7 @@
       </c>
       <c r="E55" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Заказчик: договор и гонорар</t>
+          <t xml:space="preserve">Основатели PECÀN: договор и гонорар</t>
         </is>
       </c>
       <c r="F55" s="4">
@@ -4236,7 +4236,7 @@
       </c>
       <c r="D58" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Заказчик</t>
+          <t xml:space="preserve">Основатели PECÀN</t>
         </is>
       </c>
       <c r="E58" s="3"/>
@@ -4508,7 +4508,7 @@
       </c>
       <c r="D62" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Заказчик</t>
+          <t xml:space="preserve">Основатели PECÀN</t>
         </is>
       </c>
       <c r="E62" s="3"/>
@@ -4583,7 +4583,7 @@
       </c>
       <c r="E63" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Заказчик</t>
+          <t xml:space="preserve">Основатели PECÀN</t>
         </is>
       </c>
       <c r="F63" s="4">
@@ -4653,7 +4653,7 @@
       </c>
       <c r="E64" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Заказчик, Gastro Ultima</t>
+          <t xml:space="preserve">Основатели PECÀN, Gastro Ultima</t>
         </is>
       </c>
       <c r="F64" s="4">
@@ -4718,7 +4718,7 @@
       </c>
       <c r="D65" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Заказчик</t>
+          <t xml:space="preserve">Основатели PECÀN</t>
         </is>
       </c>
       <c r="E65" s="3"/>
@@ -5250,7 +5250,7 @@
       </c>
       <c r="D73" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Заказчик</t>
+          <t xml:space="preserve">Основатели PECÀN</t>
         </is>
       </c>
       <c r="E73" s="3" t="inlineStr">
@@ -5534,7 +5534,7 @@
       </c>
       <c r="D77" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Заказчик</t>
+          <t xml:space="preserve">Основатели PECÀN</t>
         </is>
       </c>
       <c r="E77" s="3" t="inlineStr">
@@ -5675,7 +5675,7 @@
       </c>
       <c r="E79" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Заказчик: блогеры, подарочный фонд</t>
+          <t xml:space="preserve">Основатели PECÀN: блогеры, подарочный фонд</t>
         </is>
       </c>
       <c r="F79" s="4">
@@ -5740,7 +5740,7 @@
       </c>
       <c r="D80" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Заказчик</t>
+          <t xml:space="preserve">Основатели PECÀN</t>
         </is>
       </c>
       <c r="E80" s="3"/>
@@ -6167,7 +6167,7 @@
       <formula>AND($D5="Gastro Ultima",$F5&lt;=N$4+6,$G5&gt;=N$4)</formula>
     </cfRule>
     <cfRule type="expression" dxfId="1" priority="2">
-      <formula>AND($D5="Заказчик",$F5&lt;=N$4+6,$G5&gt;=N$4)</formula>
+      <formula>AND($D5="Основатели PECÀN",$F5&lt;=N$4+6,$G5&gt;=N$4)</formula>
     </cfRule>
     <cfRule type="expression" dxfId="2" priority="3">
       <formula>AND($D5="Дизайн-студия",$F5&lt;=N$4+6,$G5&gt;=N$4)</formula>
@@ -6192,7 +6192,7 @@
   </conditionalFormatting>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" sqref="D5:D125">
-      <formula1>"Gastro Ultima,Заказчик,Дизайн-студия,Строители,Поставщики и логистика,Шефы и команда"</formula1>
+      <formula1>"Gastro Ultima,Основатели PECÀN,Дизайн-студия,Строители,Поставщики и логистика,Шефы и команда"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
@@ -6294,7 +6294,7 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Заказчик</t>
+          <t xml:space="preserve">Основатели PECÀN</t>
         </is>
       </c>
       <c r="D6" s="5"/>
@@ -6319,7 +6319,7 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Заказчик</t>
+          <t xml:space="preserve">Основатели PECÀN</t>
         </is>
       </c>
       <c r="D7" s="5"/>
@@ -6365,7 +6365,7 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Заказчик</t>
+          <t xml:space="preserve">Основатели PECÀN</t>
         </is>
       </c>
       <c r="D9" s="5"/>
@@ -6436,7 +6436,7 @@
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Заказчик</t>
+          <t xml:space="preserve">Основатели PECÀN</t>
         </is>
       </c>
       <c r="D12" s="5"/>
@@ -6669,7 +6669,7 @@
     <row r="26">
       <c r="A26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Заказчик согласует материалы за 3 рабочих дня. Каждый день задержки согласования сдвигает зависимые работы.</t>
+          <t xml:space="preserve">Основатели PECÀN согласуют материалы за 3 рабочих дня. Каждый день задержки согласования сдвигает зависимые работы.</t>
         </is>
       </c>
     </row>
@@ -6760,12 +6760,12 @@
     <row r="6" ht="86" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Заказчик</t>
+          <t xml:space="preserve">Основатели PECÀN</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Инвестор и владелец</t>
+          <t xml:space="preserve">Владельцы кофейни</t>
         </is>
       </c>
       <c r="C6" s="5">
@@ -6773,11 +6773,11 @@
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">• Согласует материалы в течение 3 рабочих дней
-• Регистрирует ТОО, открывает счёт, заключает договоры
-• Оплачивает строителей, дизайн, оборудование, логистику и таможню
-• Финансирует рекламу, вывеску, полиграфию, упаковку
-• Закупает первый товарный запас и расходники</t>
+          <t xml:space="preserve">• Согласуют материалы в течение 3 рабочих дней
+• Регистрируют ТОО, открывают счёт, заключают договоры
+• Оплачивают строителей, дизайн, оборудование, логистику и таможню
+• Финансируют рекламу, вывеску, полиграфию, упаковку
+• Закупают первый товарный запас и расходники</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Single PECAN team role
</commit_message>
<xml_diff>
--- a/pecan-plan.xlsx
+++ b/pecan-plan.xlsx
@@ -286,7 +286,7 @@
     <row r="2">
       <c r="A2" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Астана, пр. Тұран, 52/4 · ведёт Gastro Ultima · состояние на 4 окт 2026 · даты, проценты и ответственных можно менять, полосы справа пересчитаются сами</t>
+          <t xml:space="preserve">Астана, пр. Тұран, 52/4 · ведёт команда PECÀN · состояние на 4 окт 2026 · даты, проценты и ответственных можно менять, полосы справа пересчитаются сами</t>
         </is>
       </c>
     </row>
@@ -454,7 +454,7 @@
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Основатели PECÀN</t>
+          <t xml:space="preserve">Команда PECÀN</t>
         </is>
       </c>
       <c r="E5" s="3"/>
@@ -520,14 +520,10 @@
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gastro Ultima</t>
-        </is>
-      </c>
-      <c r="E6" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Основатели PECÀN</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Команда PECÀN</t>
+        </is>
+      </c>
+      <c r="E6" s="3"/>
       <c r="F6" s="4">
         <v>46292</v>
       </c>
@@ -594,7 +590,7 @@
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gastro Ultima</t>
+          <t xml:space="preserve">Команда PECÀN</t>
         </is>
       </c>
       <c r="E7" s="3"/>
@@ -664,7 +660,7 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Основатели PECÀN</t>
+          <t xml:space="preserve">Команда PECÀN</t>
         </is>
       </c>
       <c r="E8" s="3"/>
@@ -734,7 +730,7 @@
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gastro Ultima</t>
+          <t xml:space="preserve">Команда PECÀN</t>
         </is>
       </c>
       <c r="E9" s="3"/>
@@ -804,7 +800,7 @@
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gastro Ultima</t>
+          <t xml:space="preserve">Команда PECÀN</t>
         </is>
       </c>
       <c r="E10" s="3"/>
@@ -874,7 +870,7 @@
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gastro Ultima</t>
+          <t xml:space="preserve">Команда PECÀN</t>
         </is>
       </c>
       <c r="E11" s="3"/>
@@ -944,7 +940,7 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gastro Ultima</t>
+          <t xml:space="preserve">Команда PECÀN</t>
         </is>
       </c>
       <c r="E12" s="3"/>
@@ -1010,14 +1006,10 @@
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gastro Ultima</t>
-        </is>
-      </c>
-      <c r="E13" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Основатели PECÀN</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Команда PECÀN</t>
+        </is>
+      </c>
+      <c r="E13" s="3"/>
       <c r="F13" s="4">
         <v>46315</v>
       </c>
@@ -1084,7 +1076,7 @@
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gastro Ultima</t>
+          <t xml:space="preserve">Команда PECÀN</t>
         </is>
       </c>
       <c r="E14" s="3"/>
@@ -1158,7 +1150,7 @@
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gastro Ultima</t>
+          <t xml:space="preserve">Команда PECÀN</t>
         </is>
       </c>
       <c r="E15" s="3"/>
@@ -1228,7 +1220,7 @@
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Основатели PECÀN</t>
+          <t xml:space="preserve">Команда PECÀN</t>
         </is>
       </c>
       <c r="E16" s="3"/>
@@ -1302,7 +1294,7 @@
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gastro Ultima</t>
+          <t xml:space="preserve">Команда PECÀN</t>
         </is>
       </c>
       <c r="E17" s="3"/>
@@ -1368,7 +1360,7 @@
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gastro Ultima</t>
+          <t xml:space="preserve">Команда PECÀN</t>
         </is>
       </c>
       <c r="E18" s="3"/>
@@ -1438,14 +1430,10 @@
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gastro Ultima</t>
-        </is>
-      </c>
-      <c r="E19" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Основатели PECÀN</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Команда PECÀN</t>
+        </is>
+      </c>
+      <c r="E19" s="3"/>
       <c r="F19" s="4">
         <v>46300</v>
       </c>
@@ -1469,7 +1457,7 @@
       </c>
       <c r="M19" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ищем с нуля. Отбор студий с опытом в кофейнях и пекарнях, сравнение сроков и стоимости, выбор вместе с основателями PECÀN. Авторский надзор включаем в договор сразу.</t>
+          <t xml:space="preserve">Ищем с нуля. Отбор студий с опытом в кофейнях и пекарнях, сравнение сроков и стоимости, выбор. Авторский надзор включаем в договор сразу.</t>
         </is>
       </c>
       <c r="N19" s="8"/>
@@ -1516,7 +1504,7 @@
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Основатели PECÀN</t>
+          <t xml:space="preserve">Команда PECÀN</t>
         </is>
       </c>
       <c r="E20" s="3"/>
@@ -1617,7 +1605,7 @@
       </c>
       <c r="M21" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Референсы от основателей PECÀN, стилистика по брендбуку, технологическое зонирование от Gastro Ultima.</t>
+          <t xml:space="preserve">Референсы команды PECÀN, стилистика по брендбуку, технологическое зонирование от команды PECÀN.</t>
         </is>
       </c>
       <c r="N21" s="8"/>
@@ -1734,7 +1722,7 @@
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gastro Ultima</t>
+          <t xml:space="preserve">Команда PECÀN</t>
         </is>
       </c>
       <c r="E23" s="3" t="inlineStr">
@@ -1952,7 +1940,7 @@
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Основатели PECÀN</t>
+          <t xml:space="preserve">Команда PECÀN</t>
         </is>
       </c>
       <c r="E26" s="3" t="inlineStr">
@@ -2099,11 +2087,7 @@
           <t xml:space="preserve">Дизайн-студия</t>
         </is>
       </c>
-      <c r="E28" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Основатели PECÀN, Gastro Ultima</t>
-        </is>
-      </c>
+      <c r="E28" s="3"/>
       <c r="F28" s="4">
         <v>46427</v>
       </c>
@@ -2170,14 +2154,10 @@
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gastro Ultima</t>
-        </is>
-      </c>
-      <c r="E29" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Основатели PECÀN</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Команда PECÀN</t>
+        </is>
+      </c>
+      <c r="E29" s="3"/>
       <c r="F29" s="4">
         <v>46300</v>
       </c>
@@ -2248,14 +2228,10 @@
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gastro Ultima</t>
-        </is>
-      </c>
-      <c r="E30" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Основатели PECÀN</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Команда PECÀN</t>
+        </is>
+      </c>
+      <c r="E30" s="3"/>
       <c r="F30" s="4">
         <v>46314</v>
       </c>
@@ -2326,7 +2302,7 @@
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Основатели PECÀN</t>
+          <t xml:space="preserve">Команда PECÀN</t>
         </is>
       </c>
       <c r="E31" s="3" t="inlineStr">
@@ -2610,7 +2586,7 @@
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gastro Ultima</t>
+          <t xml:space="preserve">Команда PECÀN</t>
         </is>
       </c>
       <c r="E35" s="3"/>
@@ -2878,12 +2854,12 @@
       </c>
       <c r="D39" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gastro Ultima</t>
+          <t xml:space="preserve">Команда PECÀN</t>
         </is>
       </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Основатели PECÀN, строители</t>
+          <t xml:space="preserve">Строители</t>
         </is>
       </c>
       <c r="F39" s="4">
@@ -3018,7 +2994,7 @@
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gastro Ultima</t>
+          <t xml:space="preserve">Команда PECÀN</t>
         </is>
       </c>
       <c r="E41" s="3"/>
@@ -3092,14 +3068,10 @@
       </c>
       <c r="D42" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gastro Ultima</t>
-        </is>
-      </c>
-      <c r="E42" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Основатели PECÀN</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Команда PECÀN</t>
+        </is>
+      </c>
+      <c r="E42" s="3"/>
       <c r="F42" s="4">
         <v>46328</v>
       </c>
@@ -3162,7 +3134,7 @@
       </c>
       <c r="D43" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gastro Ultima</t>
+          <t xml:space="preserve">Команда PECÀN</t>
         </is>
       </c>
       <c r="E43" s="3" t="inlineStr">
@@ -3240,7 +3212,7 @@
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Основатели PECÀN</t>
+          <t xml:space="preserve">Команда PECÀN</t>
         </is>
       </c>
       <c r="E44" s="3"/>
@@ -3314,14 +3286,10 @@
       </c>
       <c r="D45" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gastro Ultima</t>
-        </is>
-      </c>
-      <c r="E45" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Основатели PECÀN</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Команда PECÀN</t>
+        </is>
+      </c>
+      <c r="E45" s="3"/>
       <c r="F45" s="4">
         <v>46349</v>
       </c>
@@ -3392,14 +3360,10 @@
       </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Основатели PECÀN</t>
-        </is>
-      </c>
-      <c r="E46" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Gastro Ultima</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Команда PECÀN</t>
+        </is>
+      </c>
+      <c r="E46" s="3"/>
       <c r="F46" s="4">
         <v>46356</v>
       </c>
@@ -3466,14 +3430,10 @@
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Основатели PECÀN</t>
-        </is>
-      </c>
-      <c r="E47" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Gastro Ultima</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Команда PECÀN</t>
+        </is>
+      </c>
+      <c r="E47" s="3"/>
       <c r="F47" s="4">
         <v>46356</v>
       </c>
@@ -3829,7 +3789,7 @@
       </c>
       <c r="E52" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gastro Ultima: шеф-контроль</t>
+          <t xml:space="preserve">Команда PECÀN: шеф-контроль</t>
         </is>
       </c>
       <c r="F52" s="4">
@@ -3964,7 +3924,7 @@
       </c>
       <c r="D54" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gastro Ultima</t>
+          <t xml:space="preserve">Команда PECÀN</t>
         </is>
       </c>
       <c r="E54" s="3"/>
@@ -4030,14 +3990,10 @@
       </c>
       <c r="D55" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gastro Ultima</t>
-        </is>
-      </c>
-      <c r="E55" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Основатели PECÀN: договор и гонорар</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Команда PECÀN</t>
+        </is>
+      </c>
+      <c r="E55" s="3"/>
       <c r="F55" s="4">
         <v>46342</v>
       </c>
@@ -4100,7 +4056,7 @@
       </c>
       <c r="D56" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gastro Ultima</t>
+          <t xml:space="preserve">Команда PECÀN</t>
         </is>
       </c>
       <c r="E56" s="3"/>
@@ -4166,7 +4122,7 @@
       </c>
       <c r="D57" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gastro Ultima</t>
+          <t xml:space="preserve">Команда PECÀN</t>
         </is>
       </c>
       <c r="E57" s="3"/>
@@ -4236,7 +4192,7 @@
       </c>
       <c r="D58" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Основатели PECÀN</t>
+          <t xml:space="preserve">Команда PECÀN</t>
         </is>
       </c>
       <c r="E58" s="3"/>
@@ -4302,7 +4258,7 @@
       </c>
       <c r="D59" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gastro Ultima</t>
+          <t xml:space="preserve">Команда PECÀN</t>
         </is>
       </c>
       <c r="E59" s="3"/>
@@ -4372,7 +4328,7 @@
       </c>
       <c r="D60" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gastro Ultima</t>
+          <t xml:space="preserve">Команда PECÀN</t>
         </is>
       </c>
       <c r="E60" s="3" t="inlineStr">
@@ -4442,7 +4398,7 @@
       </c>
       <c r="D61" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Шефы и команда</t>
+          <t xml:space="preserve">Шефы и персонал</t>
         </is>
       </c>
       <c r="E61" s="3"/>
@@ -4508,7 +4464,7 @@
       </c>
       <c r="D62" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Основатели PECÀN</t>
+          <t xml:space="preserve">Команда PECÀN</t>
         </is>
       </c>
       <c r="E62" s="3"/>
@@ -4578,14 +4534,10 @@
       </c>
       <c r="D63" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gastro Ultima</t>
-        </is>
-      </c>
-      <c r="E63" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Основатели PECÀN</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Команда PECÀN</t>
+        </is>
+      </c>
+      <c r="E63" s="3"/>
       <c r="F63" s="4">
         <v>46398</v>
       </c>
@@ -4648,14 +4600,10 @@
       </c>
       <c r="D64" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Шефы и команда</t>
-        </is>
-      </c>
-      <c r="E64" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Основатели PECÀN, Gastro Ultima</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Шефы и персонал</t>
+        </is>
+      </c>
+      <c r="E64" s="3"/>
       <c r="F64" s="4">
         <v>46426</v>
       </c>
@@ -4718,7 +4666,7 @@
       </c>
       <c r="D65" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Основатели PECÀN</t>
+          <t xml:space="preserve">Команда PECÀN</t>
         </is>
       </c>
       <c r="E65" s="3"/>
@@ -4784,7 +4732,7 @@
       </c>
       <c r="D66" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gastro Ultima</t>
+          <t xml:space="preserve">Команда PECÀN</t>
         </is>
       </c>
       <c r="E66" s="3"/>
@@ -4850,7 +4798,7 @@
       </c>
       <c r="D67" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gastro Ultima</t>
+          <t xml:space="preserve">Команда PECÀN</t>
         </is>
       </c>
       <c r="E67" s="3"/>
@@ -4916,7 +4864,7 @@
       </c>
       <c r="D68" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gastro Ultima</t>
+          <t xml:space="preserve">Команда PECÀN</t>
         </is>
       </c>
       <c r="E68" s="3"/>
@@ -4982,7 +4930,7 @@
       </c>
       <c r="D69" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gastro Ultima</t>
+          <t xml:space="preserve">Команда PECÀN</t>
         </is>
       </c>
       <c r="E69" s="3"/>
@@ -5048,7 +4996,7 @@
       </c>
       <c r="D70" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gastro Ultima</t>
+          <t xml:space="preserve">Команда PECÀN</t>
         </is>
       </c>
       <c r="E70" s="3"/>
@@ -5118,7 +5066,7 @@
       </c>
       <c r="D71" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gastro Ultima</t>
+          <t xml:space="preserve">Команда PECÀN</t>
         </is>
       </c>
       <c r="E71" s="3"/>
@@ -5184,7 +5132,7 @@
       </c>
       <c r="D72" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gastro Ultima</t>
+          <t xml:space="preserve">Команда PECÀN</t>
         </is>
       </c>
       <c r="E72" s="3"/>
@@ -5250,14 +5198,10 @@
       </c>
       <c r="D73" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Основатели PECÀN</t>
-        </is>
-      </c>
-      <c r="E73" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Gastro Ultima</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Команда PECÀN</t>
+        </is>
+      </c>
+      <c r="E73" s="3"/>
       <c r="F73" s="4">
         <v>46412</v>
       </c>
@@ -5320,12 +5264,12 @@
       </c>
       <c r="D74" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gastro Ultima</t>
+          <t xml:space="preserve">Команда PECÀN</t>
         </is>
       </c>
       <c r="E74" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Команда</t>
+          <t xml:space="preserve">Персонал кофейни</t>
         </is>
       </c>
       <c r="F74" s="4">
@@ -5394,7 +5338,7 @@
       </c>
       <c r="D75" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gastro Ultima</t>
+          <t xml:space="preserve">Команда PECÀN</t>
         </is>
       </c>
       <c r="E75" s="3"/>
@@ -5468,7 +5412,7 @@
       </c>
       <c r="D76" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gastro Ultima</t>
+          <t xml:space="preserve">Команда PECÀN</t>
         </is>
       </c>
       <c r="E76" s="3"/>
@@ -5534,14 +5478,10 @@
       </c>
       <c r="D77" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Основатели PECÀN</t>
-        </is>
-      </c>
-      <c r="E77" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Gastro Ultima: медиаплан и ТЗ</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Команда PECÀN</t>
+        </is>
+      </c>
+      <c r="E77" s="3"/>
       <c r="F77" s="4">
         <v>46391</v>
       </c>
@@ -5604,7 +5544,7 @@
       </c>
       <c r="D78" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gastro Ultima</t>
+          <t xml:space="preserve">Команда PECÀN</t>
         </is>
       </c>
       <c r="E78" s="3"/>
@@ -5670,14 +5610,10 @@
       </c>
       <c r="D79" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gastro Ultima</t>
-        </is>
-      </c>
-      <c r="E79" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Основатели PECÀN: блогеры, подарочный фонд</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Команда PECÀN</t>
+        </is>
+      </c>
+      <c r="E79" s="3"/>
       <c r="F79" s="4">
         <v>46433</v>
       </c>
@@ -5740,7 +5676,7 @@
       </c>
       <c r="D80" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Основатели PECÀN</t>
+          <t xml:space="preserve">Команда PECÀN</t>
         </is>
       </c>
       <c r="E80" s="3"/>
@@ -5806,7 +5742,7 @@
       </c>
       <c r="D81" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gastro Ultima</t>
+          <t xml:space="preserve">Команда PECÀN</t>
         </is>
       </c>
       <c r="E81" s="3" t="inlineStr">
@@ -5884,12 +5820,12 @@
       </c>
       <c r="D82" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gastro Ultima</t>
+          <t xml:space="preserve">Команда PECÀN</t>
         </is>
       </c>
       <c r="E82" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Команда</t>
+          <t xml:space="preserve">Персонал кофейни</t>
         </is>
       </c>
       <c r="F82" s="4">
@@ -5962,14 +5898,10 @@
       </c>
       <c r="D83" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Шефы и команда</t>
-        </is>
-      </c>
-      <c r="E83" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Gastro Ultima</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Шефы и персонал</t>
+        </is>
+      </c>
+      <c r="E83" s="3"/>
       <c r="F83" s="4">
         <v>46443</v>
       </c>
@@ -6032,7 +5964,7 @@
       </c>
       <c r="D84" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gastro Ultima</t>
+          <t xml:space="preserve">Команда PECÀN</t>
         </is>
       </c>
       <c r="E84" s="3" t="inlineStr">
@@ -6110,7 +6042,7 @@
       </c>
       <c r="D85" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gastro Ultima</t>
+          <t xml:space="preserve">Команда PECÀN</t>
         </is>
       </c>
       <c r="E85" s="3"/>
@@ -6164,10 +6096,10 @@
   <autoFilter ref="A4:M85"/>
   <conditionalFormatting sqref="N5:AN85">
     <cfRule type="expression" dxfId="0" priority="1">
-      <formula>AND($D5="Gastro Ultima",$F5&lt;=N$4+6,$G5&gt;=N$4)</formula>
+      <formula>AND($D5="Команда PECÀN",$F5&lt;=N$4+6,$G5&gt;=N$4)</formula>
     </cfRule>
     <cfRule type="expression" dxfId="1" priority="2">
-      <formula>AND($D5="Основатели PECÀN",$F5&lt;=N$4+6,$G5&gt;=N$4)</formula>
+      <formula>AND($D5="",$F5&lt;=N$4+6,$G5&gt;=N$4)</formula>
     </cfRule>
     <cfRule type="expression" dxfId="2" priority="3">
       <formula>AND($D5="Дизайн-студия",$F5&lt;=N$4+6,$G5&gt;=N$4)</formula>
@@ -6179,7 +6111,7 @@
       <formula>AND($D5="Поставщики и логистика",$F5&lt;=N$4+6,$G5&gt;=N$4)</formula>
     </cfRule>
     <cfRule type="expression" dxfId="5" priority="6">
-      <formula>AND($D5="Шефы и команда",$F5&lt;=N$4+6,$G5&gt;=N$4)</formula>
+      <formula>AND($D5="Шефы и персонал",$F5&lt;=N$4+6,$G5&gt;=N$4)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J5:J85">
@@ -6192,7 +6124,7 @@
   </conditionalFormatting>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" sqref="D5:D125">
-      <formula1>"Gastro Ultima,Основатели PECÀN,Дизайн-студия,Строители,Поставщики и логистика,Шефы и команда"</formula1>
+      <formula1>"Команда PECÀN,Дизайн-студия,Строители,Поставщики и логистика,Шефы и персонал"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
@@ -6273,7 +6205,7 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gastro Ultima</t>
+          <t xml:space="preserve">Команда PECÀN</t>
         </is>
       </c>
       <c r="D5" s="5"/>
@@ -6294,7 +6226,7 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Основатели PECÀN</t>
+          <t xml:space="preserve">Команда PECÀN</t>
         </is>
       </c>
       <c r="D6" s="5"/>
@@ -6319,7 +6251,7 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Основатели PECÀN</t>
+          <t xml:space="preserve">Команда PECÀN</t>
         </is>
       </c>
       <c r="D7" s="5"/>
@@ -6344,7 +6276,7 @@
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gastro Ultima</t>
+          <t xml:space="preserve">Команда PECÀN</t>
         </is>
       </c>
       <c r="D8" s="5"/>
@@ -6365,7 +6297,7 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Основатели PECÀN</t>
+          <t xml:space="preserve">Команда PECÀN</t>
         </is>
       </c>
       <c r="D9" s="5"/>
@@ -6394,7 +6326,7 @@
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gastro Ultima</t>
+          <t xml:space="preserve">Команда PECÀN</t>
         </is>
       </c>
       <c r="D10" s="5"/>
@@ -6436,7 +6368,7 @@
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Основатели PECÀN</t>
+          <t xml:space="preserve">Команда PECÀN</t>
         </is>
       </c>
       <c r="D12" s="5"/>
@@ -6486,7 +6418,7 @@
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gastro Ultima</t>
+          <t xml:space="preserve">Команда PECÀN</t>
         </is>
       </c>
       <c r="D14" s="5"/>
@@ -6507,7 +6439,7 @@
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gastro Ultima</t>
+          <t xml:space="preserve">Команда PECÀN</t>
         </is>
       </c>
       <c r="D15" s="5"/>
@@ -6574,7 +6506,7 @@
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gastro Ultima</t>
+          <t xml:space="preserve">Команда PECÀN</t>
         </is>
       </c>
       <c r="D18" s="5"/>
@@ -6599,7 +6531,7 @@
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gastro Ultima</t>
+          <t xml:space="preserve">Команда PECÀN</t>
         </is>
       </c>
       <c r="D19" s="5"/>
@@ -6624,7 +6556,7 @@
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gastro Ultima</t>
+          <t xml:space="preserve">Команда PECÀN</t>
         </is>
       </c>
       <c r="D20" s="5"/>
@@ -6669,7 +6601,7 @@
     <row r="26">
       <c r="A26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Основатели PECÀN согласуют материалы за 3 рабочих дня. Каждый день задержки согласования сдвигает зависимые работы.</t>
+          <t xml:space="preserve">Материалы согласуются за 3 рабочих дня. Каждый день задержки согласования сдвигает зависимые работы.</t>
         </is>
       </c>
     </row>
@@ -6732,15 +6664,15 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="102" customHeight="1">
+    <row r="5" ht="134" customHeight="1">
       <c r="A5" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gastro Ultima</t>
+          <t xml:space="preserve">Команда PECÀN</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Консалтинг и управление проектом</t>
+          <t xml:space="preserve">Основатели и Gastro Ultima</t>
         </is>
       </c>
       <c r="C5" s="5">
@@ -6748,54 +6680,32 @@
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">• Ведёт проект целиком: график, контрольные точки, отчётность
+          <t xml:space="preserve">• Ведёт проект целиком: график, решения, согласования, бюджет
 • Аналитика локации, финансовая модель, маркетинговая стратегия
-• Технологический проект (ТХ), инженерные ТЗ, технологический надзор
-• Спецификации оснащения и выездная сессия в Китае
+• Технологический проект, инженерные ТЗ, технологический надзор
+• Выбор дизайн-студии и строительной бригады, договоры с подрядчиками
+• Спецификации, выездная сессия в Китае, оплата оборудования и логистики
+• Юрлицо, счёт, договоры с ЖКХ и поставщиками сырья
 • Подбор команды, обучение, аттестация
-• iiko, лояльность, стандарты, ХАССП, сопровождение открытия</t>
+• iiko, лояльность, стандарты, ХАССП, запуск и открытие</t>
         </is>
       </c>
     </row>
     <row r="6" ht="86" customHeight="1">
-      <c r="A6" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Основатели PECÀN</t>
+      <c r="A6" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Дизайн-студия</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Владельцы кофейни</t>
+          <t xml:space="preserve">Новый подрядчик · выбираем до 16 октября</t>
         </is>
       </c>
       <c r="C6" s="5">
         <f>COUNTIF('График'!D:D,A6)</f>
       </c>
       <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">• Согласуют материалы в течение 3 рабочих дней
-• Регистрируют ТОО, открывают счёт, заключают договоры
-• Оплачивают строителей, дизайн, оборудование, логистику и таможню
-• Финансируют рекламу, вывеску, полиграфию, упаковку
-• Закупают первый товарный запас и расходники</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="86" customHeight="1">
-      <c r="A7" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Дизайн-студия</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Новый подрядчик · выбираем до 16 октября</t>
-        </is>
-      </c>
-      <c r="C7" s="5">
-        <f>COUNTIF('График'!D:D,A7)</f>
-      </c>
-      <c r="D7" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">• Планировочное решение и концепция интерьера
 • 3D-визуализации, сверка с технологическим зонированием
@@ -6805,21 +6715,21 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="86" customHeight="1">
-      <c r="A8" s="14" t="inlineStr">
+    <row r="7" ht="86" customHeight="1">
+      <c r="A7" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">Строители</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Новая бригада · выбираем до 30 октября</t>
         </is>
       </c>
-      <c r="C8" s="5">
-        <f>COUNTIF('График'!D:D,A8)</f>
-      </c>
-      <c r="D8" s="3" t="inlineStr">
+      <c r="C7" s="5">
+        <f>COUNTIF('График'!D:D,A7)</f>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">• Черновые работы и перегородки по проекту
 • Электрика 380 В, вода, канализация, трапы, жироуловитель
@@ -6829,21 +6739,21 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="70" customHeight="1">
-      <c r="A9" s="15" t="inlineStr">
+    <row r="8" ht="70" customHeight="1">
+      <c r="A8" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">Поставщики и логистика</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Фабрики КНР, европейские линии, карго, таможня</t>
         </is>
       </c>
-      <c r="C9" s="5">
-        <f>COUNTIF('График'!D:D,A9)</f>
-      </c>
-      <c r="D9" s="3" t="inlineStr">
+      <c r="C8" s="5">
+        <f>COUNTIF('График'!D:D,A8)</f>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">• Производство мебели, света, посуды, нейтрального оборудования
 • Поставка печей, расстойки, кофемашины
@@ -6852,21 +6762,21 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="70" customHeight="1">
-      <c r="A10" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Шефы и команда</t>
-        </is>
-      </c>
-      <c r="B10" s="3" t="inlineStr">
+    <row r="9" ht="70" customHeight="1">
+      <c r="A9" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Шефы и персонал</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Шеф-пекарь, шеф-бариста, управляющий, линейный персонал</t>
         </is>
       </c>
-      <c r="C10" s="5">
-        <f>COUNTIF('График'!D:D,A10)</f>
-      </c>
-      <c r="D10" s="3" t="inlineStr">
+      <c r="C9" s="5">
+        <f>COUNTIF('График'!D:D,A9)</f>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">• Рецептуры и технологические карты
 • Проработки и дегустации меню

</xml_diff>

<commit_message>
Coffee machine from local dealer, rest from China
</commit_message>
<xml_diff>
--- a/pecan-plan.xlsx
+++ b/pecan-plan.xlsx
@@ -3425,7 +3425,7 @@
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Заказ печей, расстойки, кофемашины</t>
+          <t xml:space="preserve">Заказ кофемашины у дилера в Казахстане</t>
         </is>
       </c>
       <c r="D47" s="3" t="inlineStr">
@@ -3593,7 +3593,7 @@
       </c>
       <c r="M49" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Отгрузка с запасом до закрытия фабрик на Китайский Новый год. Как снижаем риск: Разместить заказы и внести предоплату в первую неделю после поездки, до 4 декабря.; В контракте с фабрикой указать дату готовности 8 января и удержание за просрочку.; Брать позиции из стандартных линеек с коротким сроком. Изготовление на заказ оставить только там, где без него нельзя.; Раз в неделю получать от фабрики фото и видео хода производства.; За неделю до готовности отправить на фабрику инспектора по качеству.; Печи, расстойку, кофемашину и холод покупать у дилеров в Казахстане и Европе: открытие от Китая по ним не зависит.</t>
+          <t xml:space="preserve">Отгрузка с запасом до закрытия фабрик на Китайский Новый год. Как снижаем риск: Разместить заказы и внести предоплату в первую неделю после поездки, до 4 декабря.; В контракте с фабрикой указать дату готовности 8 января и удержание за просрочку.; Брать позиции из стандартных линеек с коротким сроком. Изготовление на заказ оставить только там, где без него нельзя.; Раз в неделю получать от фабрики фото и видео хода производства.; За неделю до готовности отправить на фабрику инспектора по качеству.</t>
         </is>
       </c>
       <c r="N49" s="8"/>
@@ -6751,7 +6751,7 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Фабрики КНР, европейские линии, карго, таможня</t>
+          <t xml:space="preserve">Фабрики КНР, дилер кофемашины, карго, таможня</t>
         </is>
       </c>
       <c r="C8" s="5">
@@ -6759,8 +6759,8 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">• Производство мебели, света, посуды, нейтрального оборудования
-• Поставка печей, расстойки, кофемашины
+          <t xml:space="preserve">• Производство оборудования, мебели, света, посуды
+• Поставка кофемашины от дилера в Казахстане
 • Отгрузка до Китайского Нового года
 • Доставка, таможенное оформление, разгрузка на объекте</t>
         </is>

</xml_diff>

<commit_message>
Delivery is not a risk
</commit_message>
<xml_diff>
--- a/pecan-plan.xlsx
+++ b/pecan-plan.xlsx
@@ -3665,11 +3665,7 @@
           <t xml:space="preserve">да</t>
         </is>
       </c>
-      <c r="M50" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Сроки зависят от перевозчика и очередей на границе, повлиять на них напрямую нельзя. Как снижаем риск: Выбрать перевозчика и таможенного брокера в ноябре, до поездки. Сравнить сроки и зафиксировать их в договоре.; ТОО зарегистрировать до оплаты заказов: оно выступает импортёром.; Инвойсы, упаковочные листы и сертификаты соответствия готовить, пока идёт производство.; Разделить груз: то, без чего нельзя открыться, отправить быстрым тарифом, остальное обычным.; Застраховать груз.; Держать запас: между прибытием 29 января и открытием 15 февраля заложено две недели.</t>
-        </is>
-      </c>
+      <c r="M50" s="10"/>
       <c r="N50" s="8"/>
       <c r="O50" s="8"/>
       <c r="P50" s="8"/>

</xml_diff>

<commit_message>
Task descriptions and success criteria
</commit_message>
<xml_diff>
--- a/pecan-plan.xlsx
+++ b/pecan-plan.xlsx
@@ -353,7 +353,7 @@
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Детали и результат</t>
+          <t xml:space="preserve">Описание и результат</t>
         </is>
       </c>
       <c r="N4" s="7">
@@ -475,7 +475,11 @@
       </c>
       <c r="K5" s="5"/>
       <c r="L5" s="5"/>
-      <c r="M5" s="10"/>
+      <c r="M5" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Передача исходных материалов по проекту: заполненный бриф, обмерный план помещения 120,67 м², айдентика и брендбук. Результат: Все исходные документы лежат в общем чате, по ним можно начинать аналитику и планировку.</t>
+        </is>
+      </c>
       <c r="N5" s="8"/>
       <c r="O5" s="8"/>
       <c r="P5" s="8"/>
@@ -545,7 +549,11 @@
         </is>
       </c>
       <c r="L6" s="5"/>
-      <c r="M6" s="10"/>
+      <c r="M6" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Подписание договора на сопровождение открытия кофейни-пекарни. С этой даты идёт отсчёт всех работ. Результат: Договор подписан обеими сторонами, у каждой стороны свой экземпляр.</t>
+        </is>
+      </c>
       <c r="N6" s="8"/>
       <c r="O6" s="8"/>
       <c r="P6" s="8"/>
@@ -613,7 +621,7 @@
       <c r="L7" s="5"/>
       <c r="M7" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Перечень работ, сроки, контрольные точки и зоны ответственности. Дальше отчитываемся по нему.</t>
+          <t xml:space="preserve">Собираем все работы проекта в один график: что делаем, в какие сроки, кто отвечает, какие даты ключевые. По нему дальше отчитываемся на еженедельных созвонах. Результат: График согласован и закреплён в общем чате, все участники знают свои сроки.</t>
         </is>
       </c>
       <c r="N7" s="8"/>
@@ -683,7 +691,7 @@
       <c r="L8" s="5"/>
       <c r="M8" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Два учредителя. Упрощённая декларация выбирается сразу при регистрации. Юрлицо нужно для договоров с ЖКХ и поставщиками. После регистрации прислать реквизиты.</t>
+          <t xml:space="preserve">Регистрация ТОО на двух учредителей и открытие расчётного счёта. Основной ОКЭД 56101, режим упрощённой декларации выбирается сразу при регистрации. Юрлицо нужно для договоров с подрядчиками, поставщиками, ЖКХ и для импорта оборудования. Результат: ТОО зарегистрировано, счёт открыт, реквизиты переданы в общий чат.</t>
         </is>
       </c>
       <c r="N8" s="8"/>
@@ -753,7 +761,7 @@
       <c r="L9" s="5"/>
       <c r="M9" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Меню, средние чеки, загрузка заведений, пешеходные связи ЖК, парковки.</t>
+          <t xml:space="preserve">Обходим и изучаем кофейни и пекарни в радиусе района: меню, цены, средний чек, загрузку по времени, сильные и слабые стороны. Смотрим, чего району не хватает. Результат: Сводная таблица конкурентов и вывод: в чём PECÀN будет отличаться и какой средний чек закладывать.</t>
         </is>
       </c>
       <c r="N9" s="8"/>
@@ -823,7 +831,7 @@
       <c r="L10" s="5"/>
       <c r="M10" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Хронометраж по пр. Тұран: утро 07:30–09:30, обед 12:30–14:30, вечер 17:30–20:00, выходные. Расчёт конверсии в чеки.</t>
+          <t xml:space="preserve">Считаем людей и машины у входа в помещение на пр. Тұран в часы пик: утро 07:30–09:30, обед 12:30–14:30, вечер 17:30–20:00, отдельно выходные. По этим цифрам рассчитываем, сколько гостей и чеков реально получить в день. Результат: Отчёт с цифрами потока по часам и дням недели и расчётом ожидаемого числа чеков.</t>
         </is>
       </c>
       <c r="N10" s="8"/>
@@ -893,7 +901,7 @@
       <c r="L11" s="5"/>
       <c r="M11" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Точка безубыточности и срок окупаемости. Результат: модель в Excel и инвестиционный бюджет.</t>
+          <t xml:space="preserve">Считаем экономику проекта: сколько нужно вложить (CAPEX), ежемесячные расходы (OPEX), прогноз прибыли и убытков, движение денег по месяцам. Цифры опираются на замер трафика и анализ конкурентов. Результат: Модель в Excel с точкой безубыточности, сроком окупаемости и бюджетом открытия, который укладывается в ваш лимит.</t>
         </is>
       </c>
       <c r="N11" s="8"/>
@@ -961,7 +969,11 @@
       </c>
       <c r="K12" s="5"/>
       <c r="L12" s="5"/>
-      <c r="M12" s="10"/>
+      <c r="M12" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Формулируем, для кого PECÀN и чем он запоминается, собираем ассортиментную матрицу: категории, ценовые уровни, хиты. Продумываем механики привлечения соседей и программу лояльности. Результат: Документ со стратегией запуска и ассортиментной матрицей, с которой можно идти к шефам за меню.</t>
+        </is>
+      </c>
       <c r="N12" s="8"/>
       <c r="O12" s="8"/>
       <c r="P12" s="8"/>
@@ -1031,7 +1043,11 @@
         </is>
       </c>
       <c r="L13" s="5"/>
-      <c r="M13" s="10"/>
+      <c r="M13" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Встреча, на которой проходим финансовую модель и бюджет открытия: откуда каждая цифра и где можно сэкономить. Результат: Бюджет открытия утверждён, вопросов по цифрам не осталось.</t>
+        </is>
+      </c>
       <c r="N13" s="8"/>
       <c r="O13" s="8"/>
       <c r="P13" s="8"/>
@@ -1103,7 +1119,7 @@
       </c>
       <c r="M14" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Зал на 20–25 мест, бар и витрина, пекарня, заготовочная, мойка, склад, санузлы. Оценка антресоли при высоте 4,52 м.</t>
+          <t xml:space="preserve">Раскладываем 120 м² на зоны: зал на 20–25 мест, бар с витриной, пекарня, заготовочная, мойка, склад, санузлы. Готовим несколько вариантов и проверяем, чтобы потоки гостей, продуктов и грязной посуды не пересекались. Оцениваем антресоль при высоте потолка 4,52 м. Результат: Два–три варианта планировки с плюсами и минусами каждого, готовые к выбору.</t>
         </is>
       </c>
       <c r="N14" s="8"/>
@@ -1175,7 +1191,11 @@
           <t xml:space="preserve">да</t>
         </is>
       </c>
-      <c r="M15" s="10"/>
+      <c r="M15" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Технологический проект: чертежи с расстановкой всего оборудования и привязкой к коммуникациям, по нормам СанПиН и ХАССП. Это основной документ для строителей и для закупки оборудования. Результат: Комплект чертежей раздела ТХ, по которому можно строить и заказывать оборудование.</t>
+        </is>
+      </c>
       <c r="N15" s="8"/>
       <c r="O15" s="8"/>
       <c r="P15" s="8"/>
@@ -1249,7 +1269,11 @@
           <t xml:space="preserve">да</t>
         </is>
       </c>
-      <c r="M16" s="10"/>
+      <c r="M16" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Выбор одного варианта планировки из предложенных. От него зависят проект ТХ, дизайн и работа строителей. Результат: Вариант планировки письменно подтверждён в чате, дальше работаем только по нему.</t>
+        </is>
+      </c>
       <c r="N16" s="8"/>
       <c r="O16" s="8"/>
       <c r="P16" s="8"/>
@@ -1315,7 +1339,11 @@
       </c>
       <c r="K17" s="5"/>
       <c r="L17" s="5"/>
-      <c r="M17" s="10"/>
+      <c r="M17" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Технические задания для электриков, сантехников и вентиляционщиков: где нужны розетки и какой мощности, включая 380 В для печей, где вода, канализация, трапы и вытяжка. Результат: Три ТЗ, по которым бригада может считать смету и начинать работы.</t>
+        </is>
+      </c>
       <c r="N17" s="8"/>
       <c r="O17" s="8"/>
       <c r="P17" s="8"/>
@@ -1385,7 +1413,11 @@
         </is>
       </c>
       <c r="L18" s="5"/>
-      <c r="M18" s="10"/>
+      <c r="M18" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Передача готового раздела ТХ и инженерных ТЗ. С этого момента строители могут выходить на объект. Результат: Чертежи и ТЗ переданы, замечаний нет.</t>
+        </is>
+      </c>
       <c r="N18" s="8"/>
       <c r="O18" s="8"/>
       <c r="P18" s="8"/>
@@ -1457,7 +1489,7 @@
       </c>
       <c r="M19" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ищем с нуля. Отбор студий с опытом в кофейнях и пекарнях, сравнение сроков и стоимости, выбор. Авторский надзор включаем в договор сразу.</t>
+          <t xml:space="preserve">Ищем дизайн-студию с нуля. Отбираем студии с опытом в кофейнях и пекарнях, смотрим портфолио и реализованные объекты, запрашиваем предложения по срокам и стоимости. Авторский надзор включаем в договор сразу. Результат: Короткий список из двух–трёх студий со сравнением: стиль, сроки, стоимость, загрузка.</t>
         </is>
       </c>
       <c r="N19" s="8"/>
@@ -1533,7 +1565,11 @@
           <t xml:space="preserve">да</t>
         </is>
       </c>
-      <c r="M20" s="10"/>
+      <c r="M20" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Выбор студии и подписание договора на дизайн-проект и авторский надзор. В договоре фиксируются три даты сдачи. Результат: Договор со студией подписан, студия получила исходные материалы и приступила к работе.</t>
+        </is>
+      </c>
       <c r="N20" s="8"/>
       <c r="O20" s="8"/>
       <c r="P20" s="8"/>
@@ -1605,7 +1641,7 @@
       </c>
       <c r="M21" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Референсы команды PECÀN, стилистика по брендбуку, технологическое зонирование от команды PECÀN.</t>
+          <t xml:space="preserve">Студия предлагает образ интерьера: настроение, материалы, цвета, свет, расстановку мебели. Опирается на брендбук, референсы и утверждённое технологическое зонирование от команды PECÀN. Результат: Концепция и планировочное решение согласованы, можно делать визуализации.</t>
         </is>
       </c>
       <c r="N21" s="8"/>
@@ -1677,7 +1713,11 @@
           <t xml:space="preserve">да</t>
         </is>
       </c>
-      <c r="M22" s="10"/>
+      <c r="M22" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Реалистичные картинки будущего интерьера с основных ракурсов: вход, бар и витрина, зал, санузел. Результат: Визуализации согласованы: вы видите, как будет выглядеть кофейня, и вам это нравится.</t>
+        </is>
+      </c>
       <c r="N22" s="8"/>
       <c r="O22" s="8"/>
       <c r="P22" s="8"/>
@@ -1747,7 +1787,11 @@
       </c>
       <c r="K23" s="5"/>
       <c r="L23" s="5"/>
-      <c r="M23" s="10"/>
+      <c r="M23" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Проверяем, что красивый интерьер не ломает рабочие процессы: хватает ли места бариста, проходит ли поток гостей, помещается ли оборудование. Результат: Список правок для студии либо подтверждение, что расхождений с ТХ нет.</t>
+        </is>
+      </c>
       <c r="N23" s="8"/>
       <c r="O23" s="8"/>
       <c r="P23" s="8"/>
@@ -1819,7 +1863,7 @@
       </c>
       <c r="M24" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Рабочие чертежи, ведомости отделки, мебели и освещения, проектная смета. Срок сжатый: пять недель от договора до полного комплекта. Как снижаем риск: В договоре со студией закрепить три даты сдачи: планировка 30 октября, визуализации 6 ноября, рабочая документация 20 ноября. Оплата по этапам.; Выбирать студию с готовой командой: дизайнер, визуализатор, чертёжник. Спросить о текущей загрузке.; В первый день передать студии технологическое зонирование, брендбук и референсы.; Ведомости мебели, света и отделки получить первыми, к 13 ноября: они нужны для поездки в Китай.; Согласовывать материалы студии за 1–2 дня, а не за 3.; Строители выходят 2 ноября по проекту ТХ и не ждут дизайн.</t>
+          <t xml:space="preserve">Рабочие чертежи для строителей, ведомости отделки, мебели и освещения, проектная смета. Срок сжатый: пять недель от договора до полного комплекта. Результат: Полный комплект документации, по которому строители работают без вопросов, а мы собираем закупочные спецификации. Как снижаем риск: В договоре со студией закрепить три даты сдачи: планировка 30 октября, визуализации 6 ноября, рабочая документация 20 ноября. Оплата по этапам.; Выбирать студию с готовой командой: дизайнер, визуализатор, чертёжник. Спросить о текущей загрузке.; В первый день передать студии технологическое зонирование, брендбук и референсы.; Ведомости мебели, света и отделки получить первыми, к 13 ноября: они нужны для поездки в Китай.; Согласовывать материалы студии за 1–2 дня, а не за 3.; Строители выходят 2 ноября по проекту ТХ и не ждут дизайн.</t>
         </is>
       </c>
       <c r="N24" s="8"/>
@@ -1893,7 +1937,7 @@
       <c r="L25" s="5"/>
       <c r="M25" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Регулярные выезды на объект с выхода строителей до расстановки мебели. Проверка соответствия проекту, согласование замен материалов, ответы на вопросы бригады. Входит в договор с дизайн-студией.</t>
+          <t xml:space="preserve">Дизайнер регулярно приезжает на объект, пока идут отделка и монтаж: проверяет соответствие проекту, согласует замены материалов, отвечает на вопросы бригады. Входит в договор со студией. Результат: Интерьер построен так, как на визуализациях, отступления от проекта согласованы заранее.</t>
         </is>
       </c>
       <c r="N25" s="8"/>
@@ -1965,7 +2009,11 @@
       </c>
       <c r="K26" s="5"/>
       <c r="L26" s="5"/>
-      <c r="M26" s="10"/>
+      <c r="M26" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Фасадная вывеска по брендбуку: эскиз, согласование размещения, изготовление и монтаж. Результат: Вывеска висит на фасаде и подсвечивается, размещение согласовано.</t>
+        </is>
+      </c>
       <c r="N26" s="8"/>
       <c r="O26" s="8"/>
       <c r="P26" s="8"/>
@@ -2039,7 +2087,11 @@
           <t xml:space="preserve">да</t>
         </is>
       </c>
-      <c r="M27" s="10"/>
+      <c r="M27" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Сдача всего дизайн-проекта. Он должен быть готов до поездки в Китай, потому что по нему закупаются мебель и свет. Результат: Проект принят целиком, правок не осталось.</t>
+        </is>
+      </c>
       <c r="N27" s="8"/>
       <c r="O27" s="8"/>
       <c r="P27" s="8"/>
@@ -2109,7 +2161,11 @@
         </is>
       </c>
       <c r="L28" s="5"/>
-      <c r="M28" s="10"/>
+      <c r="M28" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Финальный обход помещения с дизайнером после расстановки мебели и декора. Результат: Дизайнер подтверждает, что интерьер соответствует проекту, список мелких доделок закрыт.</t>
+        </is>
+      </c>
       <c r="N28" s="8"/>
       <c r="O28" s="8"/>
       <c r="P28" s="8"/>
@@ -2181,7 +2237,7 @@
       </c>
       <c r="M29" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ищем с нуля. Отбор бригад с опытом в общепите: электрика 380 В, вентиляция, мокрые зоны. Выезд на их сданные объекты.</t>
+          <t xml:space="preserve">Ищем строительную бригаду с нуля. Отбираем тех, кто уже делал заведения общепита: электрика 380 В, вентиляция, мокрые зоны. Выезжаем на их сданные объекты и звоним прошлым клиентам. Результат: Три–четыре проверенные бригады, готовые дать смету.</t>
         </is>
       </c>
       <c r="N29" s="8"/>
@@ -2255,7 +2311,7 @@
       </c>
       <c r="M30" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Сметы считаются по технологическому зонированию и инженерным ТЗ, уточняются после рабочей документации дизайна.</t>
+          <t xml:space="preserve">Бригады считают сметы по нашему зонированию и инженерным ТЗ. Сравниваем цены, сроки, условия оплаты и гарантии, проверяем, что в сметах нет завышенных объёмов. Результат: Сравнительная таблица смет и рекомендация, какую бригаду брать.</t>
         </is>
       </c>
       <c r="N30" s="8"/>
@@ -2337,7 +2393,7 @@
       </c>
       <c r="M31" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">В договоре: сроки по этому графику, поэтапная оплата, закупка материалов по проектной смете.</t>
+          <t xml:space="preserve">Подписание договора подряда с выбранной бригадой. В договоре: сроки по этому графику, поэтапная оплата, закупка материалов по проектной смете. Результат: Договор подписан, бригада подтверждает выход на объект 2 ноября.</t>
         </is>
       </c>
       <c r="N31" s="8"/>
@@ -2409,7 +2465,11 @@
         </is>
       </c>
       <c r="L32" s="5"/>
-      <c r="M32" s="10"/>
+      <c r="M32" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Начало ремонта: бригада заходит на объект с материалами и инструментом. Результат: Работы на объекте начаты в срок.</t>
+        </is>
+      </c>
       <c r="N32" s="8"/>
       <c r="O32" s="8"/>
       <c r="P32" s="8"/>
@@ -2475,7 +2535,11 @@
       </c>
       <c r="K33" s="5"/>
       <c r="L33" s="5"/>
-      <c r="M33" s="10"/>
+      <c r="M33" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Разметка помещения по проекту, возведение перегородок, подготовка стен и пола под инженерные сети. Результат: Помещение разделено на зоны по планировке, перегородки стоят.</t>
+        </is>
+      </c>
       <c r="N33" s="8"/>
       <c r="O33" s="8"/>
       <c r="P33" s="8"/>
@@ -2541,7 +2605,11 @@
       </c>
       <c r="K34" s="5"/>
       <c r="L34" s="5"/>
-      <c r="M34" s="10"/>
+      <c r="M34" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Прокладка электрики с выводом 380 В под печи, водопровода, канализации, установка трапов и жироуловителя. Всё по инженерным ТЗ. Результат: Все выводы сделаны в точках по проекту и проверены до закрытия стен.</t>
+        </is>
+      </c>
       <c r="N34" s="8"/>
       <c r="O34" s="8"/>
       <c r="P34" s="8"/>
@@ -2609,7 +2677,7 @@
       <c r="L35" s="5"/>
       <c r="M35" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Акты осмотра до закрытия стен и начала чистовой отделки.</t>
+          <t xml:space="preserve">Команда PECÀN выезжает на объект и проверяет, что розетки, вода, канализация и вытяжка выведены ровно там, где будет стоять оборудование. Результат: Акты осмотра подписаны до закрытия стен, переделок после отделки не потребуется.</t>
         </is>
       </c>
       <c r="N35" s="8"/>
@@ -2677,7 +2745,11 @@
       </c>
       <c r="K36" s="5"/>
       <c r="L36" s="5"/>
-      <c r="M36" s="10"/>
+      <c r="M36" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Монтаж вытяжки над пекарней и кухней, приточной вентиляции и кондиционеров в зале. Результат: Вентиляция работает, в зале нет запахов кухни, кондиционеры охлаждают и греют.</t>
+        </is>
+      </c>
       <c r="N36" s="8"/>
       <c r="O36" s="8"/>
       <c r="P36" s="8"/>
@@ -2743,7 +2815,11 @@
       </c>
       <c r="K37" s="5"/>
       <c r="L37" s="5"/>
-      <c r="M37" s="10"/>
+      <c r="M37" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Финишная отделка стен, пола и потолка по дизайн-проекту: штукатурка, покраска, плитка, напольное покрытие. Результат: Отделка завершена и принята дизайнером, помещение выглядит как на визуализациях.</t>
+        </is>
+      </c>
       <c r="N37" s="8"/>
       <c r="O37" s="8"/>
       <c r="P37" s="8"/>
@@ -2809,7 +2885,11 @@
       </c>
       <c r="K38" s="5"/>
       <c r="L38" s="5"/>
-      <c r="M38" s="10"/>
+      <c r="M38" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Установка светильников, сантехники, барной стойки и встроенной мебели. Результат: Свет горит, вода течёт, стойка и встроенная мебель стоят на местах.</t>
+        </is>
+      </c>
       <c r="N38" s="8"/>
       <c r="O38" s="8"/>
       <c r="P38" s="8"/>
@@ -2883,7 +2963,11 @@
         </is>
       </c>
       <c r="L39" s="5"/>
-      <c r="M39" s="10"/>
+      <c r="M39" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Совместный обход помещения после ремонта: команда PECÀN, строители, дизайнер. Проверяем качество работ и готовность принять оборудование. Результат: Акт приёмки подписан, замечания устранены, помещение готово к завозу оборудования.</t>
+        </is>
+      </c>
       <c r="N39" s="8"/>
       <c r="O39" s="8"/>
       <c r="P39" s="8"/>
@@ -2949,7 +3033,11 @@
       </c>
       <c r="K40" s="5"/>
       <c r="L40" s="5"/>
-      <c r="M40" s="10"/>
+      <c r="M40" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Профессиональная уборка после строителей: пыль, следы краски, мытьё окон и полов. Результат: Помещение чистое, можно завозить оборудование и мебель.</t>
+        </is>
+      </c>
       <c r="N40" s="8"/>
       <c r="O40" s="8"/>
       <c r="P40" s="8"/>
@@ -3021,7 +3109,7 @@
       </c>
       <c r="M41" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Собираются по проекту ТХ: печи, расстойка, холод, бар, нейтральное оборудование.</t>
+          <t xml:space="preserve">Составляем точный список техники и инвентаря по проекту ТХ: печи, расстойка, холод, бар, нейтральное оборудование. Для каждой позиции указываем модель, размеры, мощность и количество. Результат: Спецификация, с которой можно ехать на фабрики и запрашивать цены.</t>
         </is>
       </c>
       <c r="N41" s="8"/>
@@ -3089,7 +3177,11 @@
       </c>
       <c r="K42" s="5"/>
       <c r="L42" s="5"/>
-      <c r="M42" s="10"/>
+      <c r="M42" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Готовим поездку: договариваемся с фабриками в Гуанчжоу и Фошане, составляем маршрут по дням, оформляем визы и покупаем билеты. Результат: Маршрут с адресами и временем встреч, визы и билеты на руках.</t>
+        </is>
+      </c>
       <c r="N42" s="8"/>
       <c r="O42" s="8"/>
       <c r="P42" s="8"/>
@@ -3165,7 +3257,7 @@
       </c>
       <c r="M43" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Собираются по ведомостям мебели и освещения из рабочей документации дизайна.</t>
+          <t xml:space="preserve">Список мебели, светильников и посуды по ведомостям из дизайн-проекта: размеры, материалы, цвета, количество. Результат: Спецификация, по которой фабрики дают цены и сроки.</t>
         </is>
       </c>
       <c r="N43" s="8"/>
@@ -3241,7 +3333,11 @@
           <t xml:space="preserve">да</t>
         </is>
       </c>
-      <c r="M44" s="10"/>
+      <c r="M44" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Утверждение списка закупок и суммы, которую готовы на них потратить. Результат: Спецификации и бюджет закупок письменно подтверждены.</t>
+        </is>
+      </c>
       <c r="N44" s="8"/>
       <c r="O44" s="8"/>
       <c r="P44" s="8"/>
@@ -3313,7 +3409,7 @@
       </c>
       <c r="M45" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Отбор посуды, мебели, света, декора и оборудования на фабриках, согласование цен.</t>
+          <t xml:space="preserve">Неделя на фабриках и в шоурумах: смотрим оборудование, мебель, свет и посуду вживую, проверяем качество, торгуемся и согласуем сроки изготовления. Результат: По каждой позиции выбран поставщик, согласованы цена и срок готовности.</t>
         </is>
       </c>
       <c r="N45" s="8"/>
@@ -3385,7 +3481,11 @@
           <t xml:space="preserve">да</t>
         </is>
       </c>
-      <c r="M46" s="10"/>
+      <c r="M46" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Подписываем контракты с фабриками и вносим предоплату. Чем раньше оплата, тем раньше фабрика запускает производство. Результат: Все заказы оплачены, фабрики подтвердили дату готовности.</t>
+        </is>
+      </c>
       <c r="N46" s="8"/>
       <c r="O46" s="8"/>
       <c r="P46" s="8"/>
@@ -3451,7 +3551,11 @@
       </c>
       <c r="K47" s="5"/>
       <c r="L47" s="5"/>
-      <c r="M47" s="10"/>
+      <c r="M47" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Выбор и заказ кофемашины у дилера в Казахстане: с гарантией, сервисом и обучением. Результат: Кофемашина оплачена, дилер подтвердил дату поставки и установки.</t>
+        </is>
+      </c>
       <c r="N47" s="8"/>
       <c r="O47" s="8"/>
       <c r="P47" s="8"/>
@@ -3521,7 +3625,11 @@
           <t xml:space="preserve">да</t>
         </is>
       </c>
-      <c r="M48" s="10"/>
+      <c r="M48" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Фабрики изготавливают заказ. Раз в неделю получаем фото и видео, чтобы видеть ход работ и сроки. Результат: Всё изготовлено к согласованной дате и соответствует образцам.</t>
+        </is>
+      </c>
       <c r="N48" s="8"/>
       <c r="O48" s="8"/>
       <c r="P48" s="8"/>
@@ -3593,7 +3701,7 @@
       </c>
       <c r="M49" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Отгрузка с запасом до закрытия фабрик на Китайский Новый год. Как снижаем риск: Разместить заказы и внести предоплату в первую неделю после поездки, до 4 декабря.; В контракте с фабрикой указать дату готовности 8 января и удержание за просрочку.; Брать позиции из стандартных линеек с коротким сроком. Изготовление на заказ оставить только там, где без него нельзя.; Раз в неделю получать от фабрики фото и видео хода производства.; За неделю до готовности отправить на фабрику инспектора по качеству.</t>
+          <t xml:space="preserve">Проверяем готовый товар на фабриках перед упаковкой и отправляем. Отгрузка с запасом до закрытия фабрик на Китайский Новый год. Результат: Товар проверен, упакован и передан перевозчику до праздников. Как снижаем риск: Разместить заказы и внести предоплату в первую неделю после поездки, до 4 декабря.; В контракте с фабрикой указать дату готовности 8 января и удержание за просрочку.; Брать позиции из стандартных линеек с коротким сроком. Изготовление на заказ оставить только там, где без него нельзя.; Раз в неделю получать от фабрики фото и видео хода производства.; За неделю до готовности отправить на фабрику инспектора по качеству.</t>
         </is>
       </c>
       <c r="N49" s="8"/>
@@ -3665,7 +3773,11 @@
           <t xml:space="preserve">да</t>
         </is>
       </c>
-      <c r="M50" s="10"/>
+      <c r="M50" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Доставка груза из Китая в Астану и таможенное оформление. Везёт наша проверенная транспортная компания. Результат: Груз растаможен и готов к доставке на объект.</t>
+        </is>
+      </c>
       <c r="N50" s="8"/>
       <c r="O50" s="8"/>
       <c r="P50" s="8"/>
@@ -3739,7 +3851,11 @@
           <t xml:space="preserve">да</t>
         </is>
       </c>
-      <c r="M51" s="10"/>
+      <c r="M51" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Разгрузка и приёмка: пересчитываем места, проверяем целостность упаковки и комплектность. Результат: Всё заказанное на объекте, повреждений нет либо они зафиксированы актом.</t>
+        </is>
+      </c>
       <c r="N51" s="8"/>
       <c r="O51" s="8"/>
       <c r="P51" s="8"/>
@@ -3813,7 +3929,11 @@
           <t xml:space="preserve">да</t>
         </is>
       </c>
-      <c r="M52" s="10"/>
+      <c r="M52" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Расстановка оборудования по проекту ТХ, подключение к электрике, воде и вытяжке, пробный запуск каждой единицы. Результат: Вся техника работает, персонал может начинать проработки.</t>
+        </is>
+      </c>
       <c r="N52" s="8"/>
       <c r="O52" s="8"/>
       <c r="P52" s="8"/>
@@ -3879,7 +3999,11 @@
       </c>
       <c r="K53" s="5"/>
       <c r="L53" s="5"/>
-      <c r="M53" s="10"/>
+      <c r="M53" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Сборка и расстановка мебели в зале, развеска светильников, декор и растения. Результат: Зал полностью обставлен и выглядит как на визуализациях.</t>
+        </is>
+      </c>
       <c r="N53" s="8"/>
       <c r="O53" s="8"/>
       <c r="P53" s="8"/>
@@ -3945,7 +4069,11 @@
       </c>
       <c r="K54" s="5"/>
       <c r="L54" s="5"/>
-      <c r="M54" s="10"/>
+      <c r="M54" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Определяем, сколько человек и на какие должности нужно, какие смены и зарплаты, как считается премия за результат. Результат: Штатное расписание с фондом оплаты труда и понятной системой мотивации.</t>
+        </is>
+      </c>
       <c r="N54" s="8"/>
       <c r="O54" s="8"/>
       <c r="P54" s="8"/>
@@ -4011,7 +4139,11 @@
       </c>
       <c r="K55" s="5"/>
       <c r="L55" s="5"/>
-      <c r="M55" s="10"/>
+      <c r="M55" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ищем шефов, которые разработают меню выпечки и кофейную карту PECÀN и обучат команду. Результат: С шеф-пекарем и шеф-бариста заключены договоры на разработку меню.</t>
+        </is>
+      </c>
       <c r="N55" s="8"/>
       <c r="O55" s="8"/>
       <c r="P55" s="8"/>
@@ -4077,7 +4209,11 @@
       </c>
       <c r="K56" s="5"/>
       <c r="L56" s="5"/>
-      <c r="M56" s="10"/>
+      <c r="M56" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ищем управляющего кофейней: размещаем вакансию, приглашаем сильных кандидатов из других заведений, проводим собеседования и проверяем рекомендации. Результат: Управляющий выбран и готов выйти на обучение 25 января.</t>
+        </is>
+      </c>
       <c r="N56" s="8"/>
       <c r="O56" s="8"/>
       <c r="P56" s="8"/>
@@ -4145,7 +4281,7 @@
       <c r="L57" s="5"/>
       <c r="M57" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Бариста, пекари, повара, кассиры, зал, клининг.</t>
+          <t xml:space="preserve">Набор команды: бариста, пекари, повара, кассиры, сотрудники зала и клининг. Вакансии, отбор анкет, собеседования, пробные смены. Результат: На каждую должность есть утверждённый кандидат с проверенными рекомендациями.</t>
         </is>
       </c>
       <c r="N57" s="8"/>
@@ -4213,7 +4349,11 @@
       </c>
       <c r="K58" s="5"/>
       <c r="L58" s="5"/>
-      <c r="M58" s="10"/>
+      <c r="M58" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Официальное оформление сотрудников и прохождение медосмотра с получением медицинских книжек. Результат: Со всеми подписаны договоры, у каждого действующая медкнижка.</t>
+        </is>
+      </c>
       <c r="N58" s="8"/>
       <c r="O58" s="8"/>
       <c r="P58" s="8"/>
@@ -4283,7 +4423,11 @@
         </is>
       </c>
       <c r="L59" s="5"/>
-      <c r="M59" s="10"/>
+      <c r="M59" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Финальная проверка: все должности закрыты, люди подтвердили выход. Результат: Полный штат из 10–14 человек готов к обучению.</t>
+        </is>
+      </c>
       <c r="N59" s="8"/>
       <c r="O59" s="8"/>
       <c r="P59" s="8"/>
@@ -4353,7 +4497,11 @@
       </c>
       <c r="K60" s="5"/>
       <c r="L60" s="5"/>
-      <c r="M60" s="10"/>
+      <c r="M60" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Определяем, что будет в меню: категории, количество позиций, фирменные хиты, завтраки, сезонные предложения. Опираемся на ассортиментную матрицу и возможности оборудования. Результат: Утверждённая структура меню, по которой шефы пишут рецептуры.</t>
+        </is>
+      </c>
       <c r="N60" s="8"/>
       <c r="O60" s="8"/>
       <c r="P60" s="8"/>
@@ -4419,7 +4567,11 @@
       </c>
       <c r="K61" s="5"/>
       <c r="L61" s="5"/>
-      <c r="M61" s="10"/>
+      <c r="M61" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Шефы разрабатывают рецепты и оформляют технологические карты: состав, граммовки, способ приготовления, себестоимость каждой позиции. Результат: На каждую позицию меню есть техкарта с себестоимостью и фото подачи.</t>
+        </is>
+      </c>
       <c r="N61" s="8"/>
       <c r="O61" s="8"/>
       <c r="P61" s="8"/>
@@ -4487,7 +4639,7 @@
       <c r="L62" s="5"/>
       <c r="M62" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">По брендбуку. Дизайн стаканов и крафтовых пакетов обновляется.</t>
+          <t xml:space="preserve">Заказ стаканов, пакетов и коробок, печать меню и ценников, пошив формы. Всё по брендбуку, дизайн стаканов и крафтовых пакетов обновляется. Результат: Упаковка, меню и форма на объекте до технического открытия.</t>
         </is>
       </c>
       <c r="N62" s="8"/>
@@ -4555,7 +4707,11 @@
       </c>
       <c r="K63" s="5"/>
       <c r="L63" s="5"/>
-      <c r="M63" s="10"/>
+      <c r="M63" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Выбираем поставщиков кофе, молока, муки, масла и остальных продуктов: сравниваем качество, цены и условия доставки, заключаем договоры. Результат: На каждый ключевой продукт есть основной и запасной поставщик с договором.</t>
+        </is>
+      </c>
       <c r="N63" s="8"/>
       <c r="O63" s="8"/>
       <c r="P63" s="8"/>
@@ -4621,7 +4777,11 @@
       </c>
       <c r="K64" s="5"/>
       <c r="L64" s="5"/>
-      <c r="M64" s="10"/>
+      <c r="M64" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Шефы готовят всё меню на нашем оборудовании, команда PECÀN пробует и даёт правки по вкусу, подаче и времени приготовления. Результат: Каждая позиция утверждена по вкусу и подаче, время отдачи укладывается в стандарт.</t>
+        </is>
+      </c>
       <c r="N64" s="8"/>
       <c r="O64" s="8"/>
       <c r="P64" s="8"/>
@@ -4687,7 +4847,11 @@
       </c>
       <c r="K65" s="5"/>
       <c r="L65" s="5"/>
-      <c r="M65" s="10"/>
+      <c r="M65" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Покупка кассовых моноблоков, принтеров чеков и лицензий iiko. Результат: Оборудование и лицензии на руках, можно начинать настройку.</t>
+        </is>
+      </c>
       <c r="N65" s="8"/>
       <c r="O65" s="8"/>
       <c r="P65" s="8"/>
@@ -4753,7 +4917,11 @@
       </c>
       <c r="K66" s="5"/>
       <c r="L66" s="5"/>
-      <c r="M66" s="10"/>
+      <c r="M66" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Настраиваем систему учёта: заносим меню, склады, техкарты шефов и правила списания продуктов. Результат: Каждая продажа автоматически списывает продукты со склада, остатки видны в системе.</t>
+        </is>
+      </c>
       <c r="N66" s="8"/>
       <c r="O66" s="8"/>
       <c r="P66" s="8"/>
@@ -4819,7 +4987,11 @@
       </c>
       <c r="K67" s="5"/>
       <c r="L67" s="5"/>
-      <c r="M67" s="10"/>
+      <c r="M67" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Настраиваем бонусную программу для гостей и связываем её с кассой, обучаем кассиров. Результат: Гость регистрируется за минуту, бонусы начисляются и списываются на кассе.</t>
+        </is>
+      </c>
       <c r="N67" s="8"/>
       <c r="O67" s="8"/>
       <c r="P67" s="8"/>
@@ -4885,7 +5057,11 @@
       </c>
       <c r="K68" s="5"/>
       <c r="L68" s="5"/>
-      <c r="M68" s="10"/>
+      <c r="M68" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Подключаем оплату через Kaspi и картой, онлайн-кассу Webkassa, принтеры на баре и кухне. Результат: Тестовая продажа проходит целиком: заказ, оплата, чек, заказ на кухне.</t>
+        </is>
+      </c>
       <c r="N68" s="8"/>
       <c r="O68" s="8"/>
       <c r="P68" s="8"/>
@@ -4951,7 +5127,11 @@
       </c>
       <c r="K69" s="5"/>
       <c r="L69" s="5"/>
-      <c r="M69" s="10"/>
+      <c r="M69" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Настраиваем отчёты, которые владельцы видят с телефона: выручка, средний чек, количество гостей, остатки. Результат: Вы открываете приложение и видите выручку за сегодня в реальном времени.</t>
+        </is>
+      </c>
       <c r="N69" s="8"/>
       <c r="O69" s="8"/>
       <c r="P69" s="8"/>
@@ -5019,7 +5199,7 @@
       <c r="L70" s="5"/>
       <c r="M70" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Решение о подключении принимают агрегаторы.</t>
+          <t xml:space="preserve">Готовим меню доставки и подаём заявки на подключение. Решение о подключении принимают сами сервисы. Результат: Заявки поданы во все четыре сервиса, меню и фото готовы.</t>
         </is>
       </c>
       <c r="N70" s="8"/>
@@ -5087,7 +5267,11 @@
       </c>
       <c r="K71" s="5"/>
       <c r="L71" s="5"/>
-      <c r="M71" s="10"/>
+      <c r="M71" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Пишем правила работы кофейни: как встречать гостя и готовить заказ, кто за что отвечает, что делать при открытии и закрытии смены, как соблюдать санитарные нормы. Результат: Комплект документов, по которым новый сотрудник понимает свою работу с первого дня.</t>
+        </is>
+      </c>
       <c r="N71" s="8"/>
       <c r="O71" s="8"/>
       <c r="P71" s="8"/>
@@ -5153,7 +5337,11 @@
       </c>
       <c r="K72" s="5"/>
       <c r="L72" s="5"/>
-      <c r="M72" s="10"/>
+      <c r="M72" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Учим управляющего вести кофейню: графики смен, заказ продуктов, себестоимость, инвентаризация, работа с отзывами и жалобами. Результат: Управляющий самостоятельно составляет график, делает заказ поставщикам и читает отчёты.</t>
+        </is>
+      </c>
       <c r="N72" s="8"/>
       <c r="O72" s="8"/>
       <c r="P72" s="8"/>
@@ -5219,7 +5407,11 @@
       </c>
       <c r="K73" s="5"/>
       <c r="L73" s="5"/>
-      <c r="M73" s="10"/>
+      <c r="M73" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Договоры на электричество, воду, вывоз мусора и дезинсекцию, уведомление о начале деятельности. Результат: Все договоры подписаны, уведомление подано, можно легально работать.</t>
+        </is>
+      </c>
       <c r="N73" s="8"/>
       <c r="O73" s="8"/>
       <c r="P73" s="8"/>
@@ -5293,7 +5485,11 @@
           <t xml:space="preserve">да</t>
         </is>
       </c>
-      <c r="M74" s="10"/>
+      <c r="M74" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Неделя обучения всей команды: бариста тренируют кофе и скорость, пекари и повара работают по техкартам, зал и касса учат меню и стандарты общения с гостем. Результат: Каждый сотрудник знает меню и свои действия на смене, готов к аттестации.</t>
+        </is>
+      </c>
       <c r="N74" s="8"/>
       <c r="O74" s="8"/>
       <c r="P74" s="8"/>
@@ -5367,7 +5563,11 @@
           <t xml:space="preserve">да</t>
         </is>
       </c>
-      <c r="M75" s="10"/>
+      <c r="M75" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Экзамен для каждого сотрудника: теория по меню и стандартам плюс практика на рабочем месте. Результат: К смене допущены только те, кто сдал аттестацию.</t>
+        </is>
+      </c>
       <c r="N75" s="8"/>
       <c r="O75" s="8"/>
       <c r="P75" s="8"/>
@@ -5433,7 +5633,11 @@
       </c>
       <c r="K76" s="5"/>
       <c r="L76" s="5"/>
-      <c r="M76" s="10"/>
+      <c r="M76" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">План продвижения: что, где и когда публикуем до и после открытия, какие активности проводим, какой бюджет на рекламу нужен. Результат: Календарь публикаций и активностей с бюджетом по неделям.</t>
+        </is>
+      </c>
       <c r="N76" s="8"/>
       <c r="O76" s="8"/>
       <c r="P76" s="8"/>
@@ -5499,7 +5703,11 @@
       </c>
       <c r="K77" s="5"/>
       <c r="L77" s="5"/>
-      <c r="M77" s="10"/>
+      <c r="M77" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ведём аккаунт до открытия: показываем ремонт, команду, пробы меню, собираем аудиторию района. Результат: К открытию у аккаунта есть живые подписчики из района, которые ждут запуска.</t>
+        </is>
+      </c>
       <c r="N77" s="8"/>
       <c r="O77" s="8"/>
       <c r="P77" s="8"/>
@@ -5565,7 +5773,11 @@
       </c>
       <c r="K78" s="5"/>
       <c r="L78" s="5"/>
-      <c r="M78" s="10"/>
+      <c r="M78" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Создаём и оформляем карточки заведения на картах: адрес, часы работы, фото, меню. Результат: PECÀN находится в поиске на картах, информация и фото актуальны.</t>
+        </is>
+      </c>
       <c r="N78" s="8"/>
       <c r="O78" s="8"/>
       <c r="P78" s="8"/>
@@ -5631,7 +5843,11 @@
       </c>
       <c r="K79" s="5"/>
       <c r="L79" s="5"/>
-      <c r="M79" s="10"/>
+      <c r="M79" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Готовим торжественное открытие: программа дня, приглашения блогерам и гостям, подарки, фото и видеосъёмка. Результат: Сценарий утверждён, гости приглашены, всё закуплено за день до события.</t>
+        </is>
+      </c>
       <c r="N79" s="8"/>
       <c r="O79" s="8"/>
       <c r="P79" s="8"/>
@@ -5697,7 +5913,11 @@
       </c>
       <c r="K80" s="5"/>
       <c r="L80" s="5"/>
-      <c r="M80" s="10"/>
+      <c r="M80" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Первая закупка продуктов, кофе, молока, упаковки и расходников под стартовое меню. Результат: Склад заполнен на первую неделю работы.</t>
+        </is>
+      </c>
       <c r="N80" s="8"/>
       <c r="O80" s="8"/>
       <c r="P80" s="8"/>
@@ -5775,7 +5995,11 @@
           <t xml:space="preserve">да</t>
         </is>
       </c>
-      <c r="M81" s="10"/>
+      <c r="M81" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Первый рабочий день без рекламы и вывески о запуске. Принимаем первых гостей и проверяем все процессы в реальной работе. Результат: Кофейня открыла двери и отработала полную смену.</t>
+        </is>
+      </c>
       <c r="N81" s="8"/>
       <c r="O81" s="8"/>
       <c r="P81" s="8"/>
@@ -5851,7 +6075,7 @@
       </c>
       <c r="M82" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Закрытая фокус-группа, калибровка скорости отдачи на пиковой нагрузке.</t>
+          <t xml:space="preserve">Десять дней работаем в тихом режиме: закрытая фокус-группа, друзья и соседи. Замеряем скорость отдачи, собираем отзывы, находим узкие места. Результат: Список проблем найден и устранён, заказ отдаётся за стандартное время даже в пик.</t>
         </is>
       </c>
       <c r="N82" s="8"/>
@@ -5919,7 +6143,11 @@
       </c>
       <c r="K83" s="5"/>
       <c r="L83" s="5"/>
-      <c r="M83" s="10"/>
+      <c r="M83" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Работаем для всех, но без громкой рекламы. Команда набирает скорость, докручиваем меню и процессы по отзывам гостей. Результат: Команда уверенно проходит пиковые часы, отзывы на картах положительные.</t>
+        </is>
+      </c>
       <c r="N83" s="8"/>
       <c r="O83" s="8"/>
       <c r="P83" s="8"/>
@@ -5997,7 +6225,11 @@
           <t xml:space="preserve">да</t>
         </is>
       </c>
-      <c r="M84" s="10"/>
+      <c r="M84" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Официальное открытие PECÀN с гостями, блогерами и праздничной программой. Результат: Праздник прошёл, о PECÀN узнал район, первые публикации вышли.</t>
+        </is>
+      </c>
       <c r="N84" s="8"/>
       <c r="O84" s="8"/>
       <c r="P84" s="8"/>
@@ -6063,7 +6295,11 @@
       </c>
       <c r="K85" s="5"/>
       <c r="L85" s="5"/>
-      <c r="M85" s="10"/>
+      <c r="M85" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Проверяем работу кофейни после открытия, передаём все документы, доступы и контакты, подписываем итоговый акт. Результат: Кофейня работает самостоятельно, у владельцев есть все документы и доступы.</t>
+        </is>
+      </c>
       <c r="N85" s="8"/>
       <c r="O85" s="8"/>
       <c r="P85" s="8"/>
@@ -6213,7 +6449,11 @@
       <c r="F5" s="5">
         <f>A5-TODAY()</f>
       </c>
-      <c r="G5" s="10"/>
+      <c r="G5" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Подписание договора на сопровождение открытия кофейни-пекарни. С этой даты идёт отсчёт всех работ.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="4">
@@ -6238,7 +6478,11 @@
       <c r="F6" s="5">
         <f>A6-TODAY()</f>
       </c>
-      <c r="G6" s="10"/>
+      <c r="G6" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Выбор одного варианта планировки из предложенных. От него зависят проект ТХ, дизайн и работа строителей.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="4">
@@ -6263,7 +6507,11 @@
       <c r="F7" s="5">
         <f>A7-TODAY()</f>
       </c>
-      <c r="G7" s="10"/>
+      <c r="G7" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Выбор студии и подписание договора на дизайн-проект и авторский надзор. В договоре фиксируются три даты сдачи.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="4">
@@ -6284,7 +6532,11 @@
       <c r="F8" s="5">
         <f>A8-TODAY()</f>
       </c>
-      <c r="G8" s="10"/>
+      <c r="G8" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Встреча, на которой проходим финансовую модель и бюджет открытия: откуда каждая цифра и где можно сэкономить.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="4">
@@ -6311,7 +6563,7 @@
       </c>
       <c r="G9" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">В договоре: сроки по этому графику, поэтапная оплата, закупка материалов по проектной смете.</t>
+          <t xml:space="preserve">Подписание договора подряда с выбранной бригадой. В договоре: сроки по этому графику, поэтапная оплата, закупка материалов по проектной смете.</t>
         </is>
       </c>
     </row>
@@ -6334,7 +6586,11 @@
       <c r="F10" s="5">
         <f>A10-TODAY()</f>
       </c>
-      <c r="G10" s="10"/>
+      <c r="G10" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Передача готового раздела ТХ и инженерных ТЗ. С этого момента строители могут выходить на объект.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="4">
@@ -6355,7 +6611,11 @@
       <c r="F11" s="5">
         <f>A11-TODAY()</f>
       </c>
-      <c r="G11" s="10"/>
+      <c r="G11" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Начало ремонта: бригада заходит на объект с материалами и инструментом.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="4">
@@ -6380,7 +6640,11 @@
       <c r="F12" s="5">
         <f>A12-TODAY()</f>
       </c>
-      <c r="G12" s="10"/>
+      <c r="G12" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Утверждение списка закупок и суммы, которую готовы на них потратить.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="4">
@@ -6405,7 +6669,11 @@
       <c r="F13" s="5">
         <f>A13-TODAY()</f>
       </c>
-      <c r="G13" s="10"/>
+      <c r="G13" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Сдача всего дизайн-проекта. Он должен быть готов до поездки в Китай, потому что по нему закупаются мебель и свет.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="4">
@@ -6426,7 +6694,11 @@
       <c r="F14" s="5">
         <f>A14-TODAY()</f>
       </c>
-      <c r="G14" s="10"/>
+      <c r="G14" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Совместный обход помещения после ремонта: команда PECÀN, строители, дизайнер. Проверяем качество работ и готовность принять оборудование.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="4">
@@ -6447,7 +6719,11 @@
       <c r="F15" s="5">
         <f>A15-TODAY()</f>
       </c>
-      <c r="G15" s="10"/>
+      <c r="G15" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Финальная проверка: все должности закрыты, люди подтвердили выход.</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="4">
@@ -6472,7 +6748,11 @@
       <c r="F16" s="5">
         <f>A16-TODAY()</f>
       </c>
-      <c r="G16" s="10"/>
+      <c r="G16" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Разгрузка и приёмка: пересчитываем места, проверяем целостность упаковки и комплектность.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="4">
@@ -6493,7 +6773,11 @@
       <c r="F17" s="5">
         <f>A17-TODAY()</f>
       </c>
-      <c r="G17" s="10"/>
+      <c r="G17" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Финальный обход помещения с дизайнером после расстановки мебели и декора.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="4">
@@ -6518,7 +6802,11 @@
       <c r="F18" s="5">
         <f>A18-TODAY()</f>
       </c>
-      <c r="G18" s="10"/>
+      <c r="G18" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Экзамен для каждого сотрудника: теория по меню и стандартам плюс практика на рабочем месте.</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="4">
@@ -6543,7 +6831,11 @@
       <c r="F19" s="5">
         <f>A19-TODAY()</f>
       </c>
-      <c r="G19" s="10"/>
+      <c r="G19" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Первый рабочий день без рекламы и вывески о запуске. Принимаем первых гостей и проверяем все процессы в реальной работе.</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="4">
@@ -6568,7 +6860,11 @@
       <c r="F20" s="5">
         <f>A20-TODAY()</f>
       </c>
-      <c r="G20" s="10"/>
+      <c r="G20" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Официальное открытие PECÀN с гостями, блогерами и праздничной программой.</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="17" t="inlineStr">

</xml_diff>

<commit_message>
Traffic count: inner alley
</commit_message>
<xml_diff>
--- a/pecan-plan.xlsx
+++ b/pecan-plan.xlsx
@@ -803,7 +803,7 @@
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Замер пешеходного и автомобильного трафика</t>
+          <t xml:space="preserve">Замер проходящего и проезжающего трафика у входа</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
@@ -831,7 +831,7 @@
       <c r="L10" s="5"/>
       <c r="M10" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Считаем людей и машины у входа в помещение на пр. Тұран в часы пик: утро 07:30–09:30, обед 12:30–14:30, вечер 17:30–20:00, отдельно выходные. По этим цифрам рассчитываем, сколько гостей и чеков реально получить в день. Результат: Отчёт с цифрами потока по часам и дням недели и расчётом ожидаемого числа чеков.</t>
+          <t xml:space="preserve">Вход в кофейню выходит на внутреннюю аллею, поэтому считаем именно её: людей, которые проходят мимо входа, и машины, которые проезжают по аллее. Припаркованные машины не учитываем. Замеры в часы пик: утро 07:30–09:30, обед 12:30–14:30, вечер 17:30–20:00, отдельно выходные. По этим цифрам рассчитываем, сколько гостей и чеков реально получить в день. Результат: Отчёт с цифрами потока по часам и дням недели и расчётом ожидаемого числа чеков.</t>
         </is>
       </c>
       <c r="N10" s="8"/>

</xml_diff>

<commit_message>
Split engineering brief and working schemes
</commit_message>
<xml_diff>
--- a/pecan-plan.xlsx
+++ b/pecan-plan.xlsx
@@ -7,7 +7,7 @@
     <sheet name="Роли" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'График'!$A$4:$M$85</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'График'!$A$4:$M$86</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'График'!$4:$4</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -1313,7 +1313,7 @@
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Инженерные ТЗ: электрика 380 В, вода, канализация, вентиляция</t>
+          <t xml:space="preserve">Задание на инженерные сети: точки подключения и нагрузки оборудования</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
@@ -1341,7 +1341,7 @@
       <c r="L17" s="5"/>
       <c r="M17" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Технические задания для электриков, сантехников и вентиляционщиков: где нужны розетки и какой мощности, включая 380 В для печей, где вода, канализация, трапы и вытяжка. Результат: Три ТЗ, по которым бригада может считать смету и начинать работы.</t>
+          <t xml:space="preserve">Команда PECÀN описывает, что нужно оборудованию: где какая розетка и какой мощности, включая 380 В для печей, где подвести воду и канализацию, где поставить трапы, какая вытяжка нужна над печами и плитой. Это задание для инженеров бригады: сами схемы и расчёты кабелей, труб и воздуховодов делают они. Результат: Задание по электрике, воде, канализации и вентиляции, по которому бригада делает рабочие схемы и считает смету.</t>
         </is>
       </c>
       <c r="N17" s="8"/>
@@ -1383,7 +1383,7 @@
       </c>
       <c r="C18" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Раздел ТХ и инженерные ТЗ сданы</t>
+          <t xml:space="preserve">Раздел ТХ и задание на инженерные сети сданы</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
@@ -1415,7 +1415,7 @@
       <c r="L18" s="5"/>
       <c r="M18" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Передача готового раздела ТХ и инженерных ТЗ. С этого момента строители могут выходить на объект. Результат: Чертежи и ТЗ переданы, замечаний нет.</t>
+          <t xml:space="preserve">Передача готового раздела ТХ и задания на инженерные сети. С этого момента строители могут выходить на объект и делать рабочие схемы. Результат: Чертежи и задание переданы, замечаний нет.</t>
         </is>
       </c>
       <c r="N18" s="8"/>
@@ -1863,7 +1863,7 @@
       </c>
       <c r="M24" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Рабочие чертежи для строителей, ведомости отделки, мебели и освещения, проектная смета. Срок сжатый: пять недель от договора до полного комплекта. Результат: Полный комплект документации, по которому строители работают без вопросов, а мы собираем закупочные спецификации. Как снижаем риск: В договоре со студией закрепить три даты сдачи: планировка 30 октября, визуализации 6 ноября, рабочая документация 20 ноября. Оплата по этапам.; Выбирать студию с готовой командой: дизайнер, визуализатор, чертёжник. Спросить о текущей загрузке.; В первый день передать студии технологическое зонирование, брендбук и референсы.; Ведомости мебели, света и отделки получить первыми, к 13 ноября: они нужны для поездки в Китай.; Согласовывать материалы студии за 1–2 дня, а не за 3.; Строители выходят 2 ноября по проекту ТХ и не ждут дизайн.</t>
+          <t xml:space="preserve">Рабочие чертежи для строителей, план освещения, план розеток и выключателей в зале, ведомости отделки, мебели и освещения, проектная смета. Срок сжатый: пять недель от договора до полного комплекта. Результат: Полный комплект документации, по которому строители работают без вопросов, а мы собираем закупочные спецификации. Как снижаем риск: В договоре со студией закрепить три даты сдачи: планировка 30 октября, визуализации 6 ноября, рабочая документация 20 ноября. Оплата по этапам.; Выбирать студию с готовой командой: дизайнер, визуализатор, чертёжник. Спросить о текущей загрузке.; В первый день передать студии технологическое зонирование, брендбук и референсы.; Ведомости мебели, света и отделки получить первыми, к 13 ноября: они нужны для поездки в Китай.; Согласовывать материалы студии за 1–2 дня, а не за 3.; Строители выходят 2 ноября по проекту ТХ и не ждут дизайн.</t>
         </is>
       </c>
       <c r="N24" s="8"/>
@@ -2237,7 +2237,7 @@
       </c>
       <c r="M29" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ищем строительную бригаду с нуля. Отбираем тех, кто уже делал заведения общепита: электрика 380 В, вентиляция, мокрые зоны. Выезжаем на их сданные объекты и звоним прошлым клиентам. Результат: Три–четыре проверенные бригады, готовые дать смету.</t>
+          <t xml:space="preserve">Ищем строительную бригаду с нуля. Отбираем тех, кто уже делал заведения общепита: электрика 380 В, вентиляция, мокрые зоны. Обязательное условие: у бригады есть свой инженер, который делает рабочие схемы сетей с расчётами. Выезжаем на сданные объекты и звоним прошлым клиентам. Результат: Три–четыре проверенные бригады, готовые дать смету.</t>
         </is>
       </c>
       <c r="N29" s="8"/>
@@ -2311,7 +2311,7 @@
       </c>
       <c r="M30" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Бригады считают сметы по нашему зонированию и инженерным ТЗ. Сравниваем цены, сроки, условия оплаты и гарантии, проверяем, что в сметах нет завышенных объёмов. Результат: Сравнительная таблица смет и рекомендация, какую бригаду брать.</t>
+          <t xml:space="preserve">Бригады считают сметы по нашему зонированию и заданию на инженерные сети. Сравниваем цены, сроки, условия оплаты и гарантии, проверяем, что в сметах нет завышенных объёмов. Результат: Сравнительная таблица смет и рекомендация, какую бригаду брать.</t>
         </is>
       </c>
       <c r="N30" s="8"/>
@@ -2509,7 +2509,7 @@
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Черновые работы и перегородки</t>
+          <t xml:space="preserve">Рабочие схемы электрики, воды и вентиляции с расчётами</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
@@ -2517,12 +2517,16 @@
           <t xml:space="preserve">Строители</t>
         </is>
       </c>
-      <c r="E33" s="3"/>
+      <c r="E33" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Команда PECÀN: проверка</t>
+        </is>
+      </c>
       <c r="F33" s="4">
         <v>46328</v>
       </c>
       <c r="G33" s="4">
-        <v>46346</v>
+        <v>46332</v>
       </c>
       <c r="H33" s="5">
         <f>G33-F33+1</f>
@@ -2537,7 +2541,7 @@
       <c r="L33" s="5"/>
       <c r="M33" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Разметка помещения по проекту, возведение перегородок, подготовка стен и пола под инженерные сети. Результат: Помещение разделено на зоны по планировке, перегородки стоят.</t>
+          <t xml:space="preserve">Инженер бригады по нашему заданию делает рабочие схемы: щит и автоматы, сечения кабелей, трассы труб, диаметры, воздуховоды и подбор вентиляторов. Розетки и свет в зале берёт из дизайн-проекта. Схемы готовы до начала прокладки сетей. Результат: Схемы электрики, водоснабжения, канализации и вентиляции проверены командой PECÀN, по ним уточнена смета.</t>
         </is>
       </c>
       <c r="N33" s="8"/>
@@ -2579,7 +2583,7 @@
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Электрика, вода, канализация, трапы, жироуловитель</t>
+          <t xml:space="preserve">Черновые работы и перегородки</t>
         </is>
       </c>
       <c r="D34" s="3" t="inlineStr">
@@ -2589,10 +2593,10 @@
       </c>
       <c r="E34" s="3"/>
       <c r="F34" s="4">
-        <v>46335</v>
+        <v>46328</v>
       </c>
       <c r="G34" s="4">
-        <v>46360</v>
+        <v>46346</v>
       </c>
       <c r="H34" s="5">
         <f>G34-F34+1</f>
@@ -2607,7 +2611,7 @@
       <c r="L34" s="5"/>
       <c r="M34" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Прокладка электрики с выводом 380 В под печи, водопровода, канализации, установка трапов и жироуловителя. Всё по инженерным ТЗ. Результат: Все выводы сделаны в точках по проекту и проверены до закрытия стен.</t>
+          <t xml:space="preserve">Разметка помещения по проекту, возведение перегородок, подготовка стен и пола под инженерные сети. Результат: Помещение разделено на зоны по планировке, перегородки стоят.</t>
         </is>
       </c>
       <c r="N34" s="8"/>
@@ -2649,12 +2653,12 @@
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Технологический надзор за выводами коммуникаций</t>
+          <t xml:space="preserve">Электрика, вода, канализация, трапы, жироуловитель</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Команда PECÀN</t>
+          <t xml:space="preserve">Строители</t>
         </is>
       </c>
       <c r="E35" s="3"/>
@@ -2662,7 +2666,7 @@
         <v>46335</v>
       </c>
       <c r="G35" s="4">
-        <v>46367</v>
+        <v>46360</v>
       </c>
       <c r="H35" s="5">
         <f>G35-F35+1</f>
@@ -2677,7 +2681,7 @@
       <c r="L35" s="5"/>
       <c r="M35" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Команда PECÀN выезжает на объект и проверяет, что розетки, вода, канализация и вытяжка выведены ровно там, где будет стоять оборудование. Результат: Акты осмотра подписаны до закрытия стен, переделок после отделки не потребуется.</t>
+          <t xml:space="preserve">Прокладка электрики с выводом 380 В под печи, водопровода, канализации, установка трапов и жироуловителя. Работы идут по рабочим схемам бригады, которые сделаны по заданию команды PECÀN. Результат: Все выводы сделаны в точках по проекту и проверены до закрытия стен.</t>
         </is>
       </c>
       <c r="N35" s="8"/>
@@ -2719,17 +2723,17 @@
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Вентиляция и кондиционирование</t>
+          <t xml:space="preserve">Технологический надзор за выводами коммуникаций</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Строители</t>
+          <t xml:space="preserve">Команда PECÀN</t>
         </is>
       </c>
       <c r="E36" s="3"/>
       <c r="F36" s="4">
-        <v>46342</v>
+        <v>46335</v>
       </c>
       <c r="G36" s="4">
         <v>46367</v>
@@ -2747,7 +2751,7 @@
       <c r="L36" s="5"/>
       <c r="M36" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Монтаж вытяжки над пекарней и кухней, приточной вентиляции и кондиционеров в зале. Результат: Вентиляция работает, в зале нет запахов кухни, кондиционеры охлаждают и греют.</t>
+          <t xml:space="preserve">Команда PECÀN выезжает на объект и проверяет, что розетки, вода, канализация и вытяжка выведены ровно там, где будет стоять оборудование, и соответствуют заданию. Результат: Акты осмотра подписаны до закрытия стен, переделок после отделки не потребуется.</t>
         </is>
       </c>
       <c r="N36" s="8"/>
@@ -2789,7 +2793,7 @@
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Чистовая отделка</t>
+          <t xml:space="preserve">Вентиляция и кондиционирование</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
@@ -2799,10 +2803,10 @@
       </c>
       <c r="E37" s="3"/>
       <c r="F37" s="4">
-        <v>46363</v>
+        <v>46342</v>
       </c>
       <c r="G37" s="4">
-        <v>46402</v>
+        <v>46367</v>
       </c>
       <c r="H37" s="5">
         <f>G37-F37+1</f>
@@ -2817,7 +2821,7 @@
       <c r="L37" s="5"/>
       <c r="M37" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Финишная отделка стен, пола и потолка по дизайн-проекту: штукатурка, покраска, плитка, напольное покрытие. Результат: Отделка завершена и принята дизайнером, помещение выглядит как на визуализациях.</t>
+          <t xml:space="preserve">Монтаж вытяжки над пекарней и кухней, приточной вентиляции и кондиционеров в зале. Результат: Вентиляция работает, в зале нет запахов кухни, кондиционеры охлаждают и греют.</t>
         </is>
       </c>
       <c r="N37" s="8"/>
@@ -2859,7 +2863,7 @@
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Свет, сантехника, столярные изделия</t>
+          <t xml:space="preserve">Чистовая отделка</t>
         </is>
       </c>
       <c r="D38" s="3" t="inlineStr">
@@ -2869,10 +2873,10 @@
       </c>
       <c r="E38" s="3"/>
       <c r="F38" s="4">
-        <v>46391</v>
+        <v>46363</v>
       </c>
       <c r="G38" s="4">
-        <v>46409</v>
+        <v>46402</v>
       </c>
       <c r="H38" s="5">
         <f>G38-F38+1</f>
@@ -2887,7 +2891,7 @@
       <c r="L38" s="5"/>
       <c r="M38" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Установка светильников, сантехники, барной стойки и встроенной мебели. Результат: Свет горит, вода течёт, стойка и встроенная мебель стоят на местах.</t>
+          <t xml:space="preserve">Финишная отделка стен, пола и потолка по дизайн-проекту: штукатурка, покраска, плитка, напольное покрытие. Результат: Отделка завершена и принята дизайнером, помещение выглядит как на визуализациях.</t>
         </is>
       </c>
       <c r="N38" s="8"/>
@@ -2927,26 +2931,22 @@
           <t xml:space="preserve">Строительство и отделка</t>
         </is>
       </c>
-      <c r="C39" s="17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Приёмка строительной готовности</t>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Свет, сантехника, столярные изделия</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Команда PECÀN</t>
-        </is>
-      </c>
-      <c r="E39" s="3" t="inlineStr">
-        <is>
           <t xml:space="preserve">Строители</t>
         </is>
       </c>
+      <c r="E39" s="3"/>
       <c r="F39" s="4">
-        <v>46412</v>
+        <v>46391</v>
       </c>
       <c r="G39" s="4">
-        <v>46412</v>
+        <v>46409</v>
       </c>
       <c r="H39" s="5">
         <f>G39-F39+1</f>
@@ -2957,15 +2957,11 @@
       <c r="J39" s="5" t="str">
         <f>IF(I39&gt;=1,"Готово",IF(G39&lt;TODAY(),"Просрочено",IF(F39&lt;=TODAY(),"В работе","В плане")))</f>
       </c>
-      <c r="K39" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">да</t>
-        </is>
-      </c>
+      <c r="K39" s="5"/>
       <c r="L39" s="5"/>
       <c r="M39" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Совместный обход помещения после ремонта: команда PECÀN, строители, дизайнер. Проверяем качество работ и готовность принять оборудование. Результат: Акт приёмки подписан, замечания устранены, помещение готово к завозу оборудования.</t>
+          <t xml:space="preserve">Установка светильников, сантехники, барной стойки и встроенной мебели. Результат: Свет горит, вода течёт, стойка и встроенная мебель стоят на местах.</t>
         </is>
       </c>
       <c r="N39" s="8"/>
@@ -3005,22 +3001,26 @@
           <t xml:space="preserve">Строительство и отделка</t>
         </is>
       </c>
-      <c r="C40" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Генеральная уборка после ремонта</t>
+      <c r="C40" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Приёмка строительной готовности</t>
         </is>
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
+          <t xml:space="preserve">Команда PECÀN</t>
+        </is>
+      </c>
+      <c r="E40" s="3" t="inlineStr">
+        <is>
           <t xml:space="preserve">Строители</t>
         </is>
       </c>
-      <c r="E40" s="3"/>
       <c r="F40" s="4">
         <v>46412</v>
       </c>
       <c r="G40" s="4">
-        <v>46414</v>
+        <v>46412</v>
       </c>
       <c r="H40" s="5">
         <f>G40-F40+1</f>
@@ -3031,11 +3031,15 @@
       <c r="J40" s="5" t="str">
         <f>IF(I40&gt;=1,"Готово",IF(G40&lt;TODAY(),"Просрочено",IF(F40&lt;=TODAY(),"В работе","В плане")))</f>
       </c>
-      <c r="K40" s="5"/>
+      <c r="K40" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">да</t>
+        </is>
+      </c>
       <c r="L40" s="5"/>
       <c r="M40" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Профессиональная уборка после строителей: пыль, следы краски, мытьё окон и полов. Результат: Помещение чистое, можно завозить оборудование и мебель.</t>
+          <t xml:space="preserve">Совместный обход помещения после ремонта: команда PECÀN, строители, дизайнер. Проверяем качество работ и готовность принять оборудование. Результат: Акт приёмки подписан, замечания устранены, помещение готово к завозу оборудования.</t>
         </is>
       </c>
       <c r="N40" s="8"/>
@@ -3072,25 +3076,25 @@
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Комплектация и Китай</t>
+          <t xml:space="preserve">Строительство и отделка</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Спецификации технологического оборудования и инвентаря</t>
+          <t xml:space="preserve">Генеральная уборка после ремонта</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Команда PECÀN</t>
+          <t xml:space="preserve">Строители</t>
         </is>
       </c>
       <c r="E41" s="3"/>
       <c r="F41" s="4">
-        <v>46321</v>
+        <v>46412</v>
       </c>
       <c r="G41" s="4">
-        <v>46339</v>
+        <v>46414</v>
       </c>
       <c r="H41" s="5">
         <f>G41-F41+1</f>
@@ -3102,14 +3106,10 @@
         <f>IF(I41&gt;=1,"Готово",IF(G41&lt;TODAY(),"Просрочено",IF(F41&lt;=TODAY(),"В работе","В плане")))</f>
       </c>
       <c r="K41" s="5"/>
-      <c r="L41" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">да</t>
-        </is>
-      </c>
+      <c r="L41" s="5"/>
       <c r="M41" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Составляем точный список техники и инвентаря по проекту ТХ: печи, расстойка, холод, бар, нейтральное оборудование. Для каждой позиции указываем модель, размеры, мощность и количество. Результат: Спецификация, с которой можно ехать на фабрики и запрашивать цены.</t>
+          <t xml:space="preserve">Профессиональная уборка после строителей: пыль, следы краски, мытьё окон и полов. Результат: Помещение чистое, можно завозить оборудование и мебель.</t>
         </is>
       </c>
       <c r="N41" s="8"/>
@@ -3151,7 +3151,7 @@
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Подготовка поездки: маршрут фабрик, визы, билеты</t>
+          <t xml:space="preserve">Спецификации технологического оборудования и инвентаря</t>
         </is>
       </c>
       <c r="D42" s="3" t="inlineStr">
@@ -3161,10 +3161,10 @@
       </c>
       <c r="E42" s="3"/>
       <c r="F42" s="4">
-        <v>46328</v>
+        <v>46321</v>
       </c>
       <c r="G42" s="4">
-        <v>46346</v>
+        <v>46339</v>
       </c>
       <c r="H42" s="5">
         <f>G42-F42+1</f>
@@ -3176,10 +3176,14 @@
         <f>IF(I42&gt;=1,"Готово",IF(G42&lt;TODAY(),"Просрочено",IF(F42&lt;=TODAY(),"В работе","В плане")))</f>
       </c>
       <c r="K42" s="5"/>
-      <c r="L42" s="5"/>
+      <c r="L42" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">да</t>
+        </is>
+      </c>
       <c r="M42" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Готовим поездку: договариваемся с фабриками в Гуанчжоу и Фошане, составляем маршрут по дням, оформляем визы и покупаем билеты. Результат: Маршрут с адресами и временем встреч, визы и билеты на руках.</t>
+          <t xml:space="preserve">Составляем точный список техники и инвентаря по проекту ТХ: печи, расстойка, холод, бар, нейтральное оборудование. Для каждой позиции указываем модель, размеры, мощность и количество. Результат: Спецификация, с которой можно ехать на фабрики и запрашивать цены.</t>
         </is>
       </c>
       <c r="N42" s="8"/>
@@ -3221,7 +3225,7 @@
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Спецификации мебели, света и посуды по дизайн-проекту</t>
+          <t xml:space="preserve">Подготовка поездки: маршрут фабрик, визы, билеты</t>
         </is>
       </c>
       <c r="D43" s="3" t="inlineStr">
@@ -3229,13 +3233,9 @@
           <t xml:space="preserve">Команда PECÀN</t>
         </is>
       </c>
-      <c r="E43" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Дизайн-студия</t>
-        </is>
-      </c>
+      <c r="E43" s="3"/>
       <c r="F43" s="4">
-        <v>46335</v>
+        <v>46328</v>
       </c>
       <c r="G43" s="4">
         <v>46346</v>
@@ -3250,14 +3250,10 @@
         <f>IF(I43&gt;=1,"Готово",IF(G43&lt;TODAY(),"Просрочено",IF(F43&lt;=TODAY(),"В работе","В плане")))</f>
       </c>
       <c r="K43" s="5"/>
-      <c r="L43" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">да</t>
-        </is>
-      </c>
+      <c r="L43" s="5"/>
       <c r="M43" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Список мебели, светильников и посуды по ведомостям из дизайн-проекта: размеры, материалы, цвета, количество. Результат: Спецификация, по которой фабрики дают цены и сроки.</t>
+          <t xml:space="preserve">Готовим поездку: договариваемся с фабриками в Гуанчжоу и Фошане, составляем маршрут по дням, оформляем визы и покупаем билеты. Результат: Маршрут с адресами и временем встреч, визы и билеты на руках.</t>
         </is>
       </c>
       <c r="N43" s="8"/>
@@ -3297,9 +3293,9 @@
           <t xml:space="preserve">Комплектация и Китай</t>
         </is>
       </c>
-      <c r="C44" s="17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Спецификации и бюджет закупок утверждены</t>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Спецификации мебели, света и посуды по дизайн-проекту</t>
         </is>
       </c>
       <c r="D44" s="3" t="inlineStr">
@@ -3307,9 +3303,13 @@
           <t xml:space="preserve">Команда PECÀN</t>
         </is>
       </c>
-      <c r="E44" s="3"/>
+      <c r="E44" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Дизайн-студия</t>
+        </is>
+      </c>
       <c r="F44" s="4">
-        <v>46346</v>
+        <v>46335</v>
       </c>
       <c r="G44" s="4">
         <v>46346</v>
@@ -3323,19 +3323,15 @@
       <c r="J44" s="5" t="str">
         <f>IF(I44&gt;=1,"Готово",IF(G44&lt;TODAY(),"Просрочено",IF(F44&lt;=TODAY(),"В работе","В плане")))</f>
       </c>
-      <c r="K44" s="5" t="inlineStr">
+      <c r="K44" s="5"/>
+      <c r="L44" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">да</t>
         </is>
       </c>
-      <c r="L44" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">да</t>
-        </is>
-      </c>
       <c r="M44" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Утверждение списка закупок и суммы, которую готовы на них потратить. Результат: Спецификации и бюджет закупок письменно подтверждены.</t>
+          <t xml:space="preserve">Список мебели, светильников и посуды по ведомостям из дизайн-проекта: размеры, материалы, цвета, количество. Результат: Спецификация, по которой фабрики дают цены и сроки.</t>
         </is>
       </c>
       <c r="N44" s="8"/>
@@ -3375,9 +3371,9 @@
           <t xml:space="preserve">Комплектация и Китай</t>
         </is>
       </c>
-      <c r="C45" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Выездная сессия в Китае: Гуанчжоу, Фошань</t>
+      <c r="C45" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Спецификации и бюджет закупок утверждены</t>
         </is>
       </c>
       <c r="D45" s="3" t="inlineStr">
@@ -3387,10 +3383,10 @@
       </c>
       <c r="E45" s="3"/>
       <c r="F45" s="4">
-        <v>46349</v>
+        <v>46346</v>
       </c>
       <c r="G45" s="4">
-        <v>46355</v>
+        <v>46346</v>
       </c>
       <c r="H45" s="5">
         <f>G45-F45+1</f>
@@ -3401,7 +3397,11 @@
       <c r="J45" s="5" t="str">
         <f>IF(I45&gt;=1,"Готово",IF(G45&lt;TODAY(),"Просрочено",IF(F45&lt;=TODAY(),"В работе","В плане")))</f>
       </c>
-      <c r="K45" s="5"/>
+      <c r="K45" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">да</t>
+        </is>
+      </c>
       <c r="L45" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">да</t>
@@ -3409,7 +3409,7 @@
       </c>
       <c r="M45" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Неделя на фабриках и в шоурумах: смотрим оборудование, мебель, свет и посуду вживую, проверяем качество, торгуемся и согласуем сроки изготовления. Результат: По каждой позиции выбран поставщик, согласованы цена и срок готовности.</t>
+          <t xml:space="preserve">Утверждение списка закупок и суммы, которую готовы на них потратить. Результат: Спецификации и бюджет закупок письменно подтверждены.</t>
         </is>
       </c>
       <c r="N45" s="8"/>
@@ -3451,7 +3451,7 @@
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Размещение заказов и предоплата фабрикам</t>
+          <t xml:space="preserve">Выездная сессия в Китае: Гуанчжоу, Фошань</t>
         </is>
       </c>
       <c r="D46" s="3" t="inlineStr">
@@ -3461,10 +3461,10 @@
       </c>
       <c r="E46" s="3"/>
       <c r="F46" s="4">
-        <v>46356</v>
+        <v>46349</v>
       </c>
       <c r="G46" s="4">
-        <v>46360</v>
+        <v>46355</v>
       </c>
       <c r="H46" s="5">
         <f>G46-F46+1</f>
@@ -3483,7 +3483,7 @@
       </c>
       <c r="M46" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Подписываем контракты с фабриками и вносим предоплату. Чем раньше оплата, тем раньше фабрика запускает производство. Результат: Все заказы оплачены, фабрики подтвердили дату готовности.</t>
+          <t xml:space="preserve">Неделя на фабриках и в шоурумах: смотрим оборудование, мебель, свет и посуду вживую, проверяем качество, торгуемся и согласуем сроки изготовления. Результат: По каждой позиции выбран поставщик, согласованы цена и срок готовности.</t>
         </is>
       </c>
       <c r="N46" s="8"/>
@@ -3525,7 +3525,7 @@
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Заказ кофемашины у дилера в Казахстане</t>
+          <t xml:space="preserve">Размещение заказов и предоплата фабрикам</t>
         </is>
       </c>
       <c r="D47" s="3" t="inlineStr">
@@ -3538,7 +3538,7 @@
         <v>46356</v>
       </c>
       <c r="G47" s="4">
-        <v>46367</v>
+        <v>46360</v>
       </c>
       <c r="H47" s="5">
         <f>G47-F47+1</f>
@@ -3550,10 +3550,14 @@
         <f>IF(I47&gt;=1,"Готово",IF(G47&lt;TODAY(),"Просрочено",IF(F47&lt;=TODAY(),"В работе","В плане")))</f>
       </c>
       <c r="K47" s="5"/>
-      <c r="L47" s="5"/>
+      <c r="L47" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">да</t>
+        </is>
+      </c>
       <c r="M47" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Выбор и заказ кофемашины у дилера в Казахстане: с гарантией, сервисом и обучением. Результат: Кофемашина оплачена, дилер подтвердил дату поставки и установки.</t>
+          <t xml:space="preserve">Подписываем контракты с фабриками и вносим предоплату. Чем раньше оплата, тем раньше фабрика запускает производство. Результат: Все заказы оплачены, фабрики подтвердили дату готовности.</t>
         </is>
       </c>
       <c r="N47" s="8"/>
@@ -3595,20 +3599,20 @@
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Производство на фабриках</t>
+          <t xml:space="preserve">Заказ кофемашины у дилера в Казахстане</t>
         </is>
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Поставщики и логистика</t>
+          <t xml:space="preserve">Команда PECÀN</t>
         </is>
       </c>
       <c r="E48" s="3"/>
       <c r="F48" s="4">
-        <v>46363</v>
+        <v>46356</v>
       </c>
       <c r="G48" s="4">
-        <v>46395</v>
+        <v>46367</v>
       </c>
       <c r="H48" s="5">
         <f>G48-F48+1</f>
@@ -3620,14 +3624,10 @@
         <f>IF(I48&gt;=1,"Готово",IF(G48&lt;TODAY(),"Просрочено",IF(F48&lt;=TODAY(),"В работе","В плане")))</f>
       </c>
       <c r="K48" s="5"/>
-      <c r="L48" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">да</t>
-        </is>
-      </c>
+      <c r="L48" s="5"/>
       <c r="M48" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Фабрики изготавливают заказ. Раз в неделю получаем фото и видео, чтобы видеть ход работ и сроки. Результат: Всё изготовлено к согласованной дате и соответствует образцам.</t>
+          <t xml:space="preserve">Выбор и заказ кофемашины у дилера в Казахстане: с гарантией, сервисом и обучением. Результат: Кофемашина оплачена, дилер подтвердил дату поставки и установки.</t>
         </is>
       </c>
       <c r="N48" s="8"/>
@@ -3669,7 +3669,7 @@
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Контроль качества и отгрузка из Китая</t>
+          <t xml:space="preserve">Производство на фабриках</t>
         </is>
       </c>
       <c r="D49" s="3" t="inlineStr">
@@ -3679,10 +3679,10 @@
       </c>
       <c r="E49" s="3"/>
       <c r="F49" s="4">
-        <v>46391</v>
+        <v>46363</v>
       </c>
       <c r="G49" s="4">
-        <v>46400</v>
+        <v>46395</v>
       </c>
       <c r="H49" s="5">
         <f>G49-F49+1</f>
@@ -3701,7 +3701,7 @@
       </c>
       <c r="M49" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Проверяем готовый товар на фабриках перед упаковкой и отправляем. Отгрузка с запасом до закрытия фабрик на Китайский Новый год. Результат: Товар проверен, упакован и передан перевозчику до праздников. Как снижаем риск: Разместить заказы и внести предоплату в первую неделю после поездки, до 4 декабря.; В контракте с фабрикой указать дату готовности 8 января и удержание за просрочку.; Брать позиции из стандартных линеек с коротким сроком. Изготовление на заказ оставить только там, где без него нельзя.; Раз в неделю получать от фабрики фото и видео хода производства.; За неделю до готовности отправить на фабрику инспектора по качеству.</t>
+          <t xml:space="preserve">Фабрики изготавливают заказ. Раз в неделю получаем фото и видео, чтобы видеть ход работ и сроки. Результат: Всё изготовлено к согласованной дате и соответствует образцам.</t>
         </is>
       </c>
       <c r="N49" s="8"/>
@@ -3743,7 +3743,7 @@
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Доставка и таможенное оформление</t>
+          <t xml:space="preserve">Контроль качества и отгрузка из Китая</t>
         </is>
       </c>
       <c r="D50" s="3" t="inlineStr">
@@ -3753,10 +3753,10 @@
       </c>
       <c r="E50" s="3"/>
       <c r="F50" s="4">
+        <v>46391</v>
+      </c>
+      <c r="G50" s="4">
         <v>46400</v>
-      </c>
-      <c r="G50" s="4">
-        <v>46416</v>
       </c>
       <c r="H50" s="5">
         <f>G50-F50+1</f>
@@ -3775,7 +3775,7 @@
       </c>
       <c r="M50" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Доставка груза из Китая в Астану и таможенное оформление. Везёт наша проверенная транспортная компания. Результат: Груз растаможен и готов к доставке на объект.</t>
+          <t xml:space="preserve">Проверяем готовый товар на фабриках перед упаковкой и отправляем. Отгрузка с запасом до закрытия фабрик на Китайский Новый год. Результат: Товар проверен, упакован и передан перевозчику до праздников. Как снижаем риск: Разместить заказы и внести предоплату в первую неделю после поездки, до 4 декабря.; В контракте с фабрикой указать дату готовности 8 января и удержание за просрочку.; Брать позиции из стандартных линеек с коротким сроком. Изготовление на заказ оставить только там, где без него нельзя.; Раз в неделю получать от фабрики фото и видео хода производства.; За неделю до готовности отправить на фабрику инспектора по качеству.</t>
         </is>
       </c>
       <c r="N50" s="8"/>
@@ -3815,9 +3815,9 @@
           <t xml:space="preserve">Комплектация и Китай</t>
         </is>
       </c>
-      <c r="C51" s="17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Оборудование и мебель на объекте</t>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Доставка и таможенное оформление</t>
         </is>
       </c>
       <c r="D51" s="3" t="inlineStr">
@@ -3827,7 +3827,7 @@
       </c>
       <c r="E51" s="3"/>
       <c r="F51" s="4">
-        <v>46416</v>
+        <v>46400</v>
       </c>
       <c r="G51" s="4">
         <v>46416</v>
@@ -3841,19 +3841,15 @@
       <c r="J51" s="5" t="str">
         <f>IF(I51&gt;=1,"Готово",IF(G51&lt;TODAY(),"Просрочено",IF(F51&lt;=TODAY(),"В работе","В плане")))</f>
       </c>
-      <c r="K51" s="5" t="inlineStr">
+      <c r="K51" s="5"/>
+      <c r="L51" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">да</t>
         </is>
       </c>
-      <c r="L51" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">да</t>
-        </is>
-      </c>
       <c r="M51" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Разгрузка и приёмка: пересчитываем места, проверяем целостность упаковки и комплектность. Результат: Всё заказанное на объекте, повреждений нет либо они зафиксированы актом.</t>
+          <t xml:space="preserve">Доставка груза из Китая в Астану и таможенное оформление. Везёт наша проверенная транспортная компания. Результат: Груз растаможен и готов к доставке на объект.</t>
         </is>
       </c>
       <c r="N51" s="8"/>
@@ -3893,9 +3889,9 @@
           <t xml:space="preserve">Комплектация и Китай</t>
         </is>
       </c>
-      <c r="C52" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Монтаж оборудования, пусконаладка</t>
+      <c r="C52" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Оборудование и мебель на объекте</t>
         </is>
       </c>
       <c r="D52" s="3" t="inlineStr">
@@ -3903,16 +3899,12 @@
           <t xml:space="preserve">Поставщики и логистика</t>
         </is>
       </c>
-      <c r="E52" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Команда PECÀN: шеф-контроль</t>
-        </is>
-      </c>
+      <c r="E52" s="3"/>
       <c r="F52" s="4">
-        <v>46419</v>
+        <v>46416</v>
       </c>
       <c r="G52" s="4">
-        <v>46425</v>
+        <v>46416</v>
       </c>
       <c r="H52" s="5">
         <f>G52-F52+1</f>
@@ -3923,7 +3915,11 @@
       <c r="J52" s="5" t="str">
         <f>IF(I52&gt;=1,"Готово",IF(G52&lt;TODAY(),"Просрочено",IF(F52&lt;=TODAY(),"В работе","В плане")))</f>
       </c>
-      <c r="K52" s="5"/>
+      <c r="K52" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">да</t>
+        </is>
+      </c>
       <c r="L52" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">да</t>
@@ -3931,7 +3927,7 @@
       </c>
       <c r="M52" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Расстановка оборудования по проекту ТХ, подключение к электрике, воде и вытяжке, пробный запуск каждой единицы. Результат: Вся техника работает, персонал может начинать проработки.</t>
+          <t xml:space="preserve">Разгрузка и приёмка: пересчитываем места, проверяем целостность упаковки и комплектность. Результат: Всё заказанное на объекте, повреждений нет либо они зафиксированы актом.</t>
         </is>
       </c>
       <c r="N52" s="8"/>
@@ -3973,20 +3969,24 @@
       </c>
       <c r="C53" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Расстановка мебели, свет, декор</t>
+          <t xml:space="preserve">Монтаж оборудования, пусконаладка</t>
         </is>
       </c>
       <c r="D53" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Дизайн-студия</t>
-        </is>
-      </c>
-      <c r="E53" s="3"/>
+          <t xml:space="preserve">Поставщики и логистика</t>
+        </is>
+      </c>
+      <c r="E53" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Команда PECÀN: шеф-контроль</t>
+        </is>
+      </c>
       <c r="F53" s="4">
-        <v>46421</v>
+        <v>46419</v>
       </c>
       <c r="G53" s="4">
-        <v>46427</v>
+        <v>46425</v>
       </c>
       <c r="H53" s="5">
         <f>G53-F53+1</f>
@@ -3998,10 +3998,14 @@
         <f>IF(I53&gt;=1,"Готово",IF(G53&lt;TODAY(),"Просрочено",IF(F53&lt;=TODAY(),"В работе","В плане")))</f>
       </c>
       <c r="K53" s="5"/>
-      <c r="L53" s="5"/>
+      <c r="L53" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">да</t>
+        </is>
+      </c>
       <c r="M53" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Сборка и расстановка мебели в зале, развеска светильников, декор и растения. Результат: Зал полностью обставлен и выглядит как на визуализациях.</t>
+          <t xml:space="preserve">Расстановка оборудования по проекту ТХ, подключение к электрике, воде и вытяжке, пробный запуск каждой единицы. Результат: Вся техника работает, персонал может начинать проработки.</t>
         </is>
       </c>
       <c r="N53" s="8"/>
@@ -4038,25 +4042,25 @@
       </c>
       <c r="B54" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Команда</t>
+          <t xml:space="preserve">Комплектация и Китай</t>
         </is>
       </c>
       <c r="C54" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Штатное расписание, фонд оплаты труда, KPI</t>
+          <t xml:space="preserve">Расстановка мебели, свет, декор</t>
         </is>
       </c>
       <c r="D54" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Команда PECÀN</t>
+          <t xml:space="preserve">Дизайн-студия</t>
         </is>
       </c>
       <c r="E54" s="3"/>
       <c r="F54" s="4">
-        <v>46328</v>
+        <v>46421</v>
       </c>
       <c r="G54" s="4">
-        <v>46339</v>
+        <v>46427</v>
       </c>
       <c r="H54" s="5">
         <f>G54-F54+1</f>
@@ -4071,7 +4075,7 @@
       <c r="L54" s="5"/>
       <c r="M54" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Определяем, сколько человек и на какие должности нужно, какие смены и зарплаты, как считается премия за результат. Результат: Штатное расписание с фондом оплаты труда и понятной системой мотивации.</t>
+          <t xml:space="preserve">Сборка и расстановка мебели в зале, развеска светильников, декор и растения. Результат: Зал полностью обставлен и выглядит как на визуализациях.</t>
         </is>
       </c>
       <c r="N54" s="8"/>
@@ -4113,7 +4117,7 @@
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Подбор шеф-пекаря и шеф-бариста</t>
+          <t xml:space="preserve">Штатное расписание, фонд оплаты труда, KPI</t>
         </is>
       </c>
       <c r="D55" s="3" t="inlineStr">
@@ -4123,10 +4127,10 @@
       </c>
       <c r="E55" s="3"/>
       <c r="F55" s="4">
-        <v>46342</v>
+        <v>46328</v>
       </c>
       <c r="G55" s="4">
-        <v>46367</v>
+        <v>46339</v>
       </c>
       <c r="H55" s="5">
         <f>G55-F55+1</f>
@@ -4141,7 +4145,7 @@
       <c r="L55" s="5"/>
       <c r="M55" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ищем шефов, которые разработают меню выпечки и кофейную карту PECÀN и обучат команду. Результат: С шеф-пекарем и шеф-бариста заключены договоры на разработку меню.</t>
+          <t xml:space="preserve">Определяем, сколько человек и на какие должности нужно, какие смены и зарплаты, как считается премия за результат. Результат: Штатное расписание с фондом оплаты труда и понятной системой мотивации.</t>
         </is>
       </c>
       <c r="N55" s="8"/>
@@ -4183,7 +4187,7 @@
       </c>
       <c r="C56" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Поиск управляющего</t>
+          <t xml:space="preserve">Подбор шеф-пекаря и шеф-бариста</t>
         </is>
       </c>
       <c r="D56" s="3" t="inlineStr">
@@ -4196,7 +4200,7 @@
         <v>46342</v>
       </c>
       <c r="G56" s="4">
-        <v>46374</v>
+        <v>46367</v>
       </c>
       <c r="H56" s="5">
         <f>G56-F56+1</f>
@@ -4211,7 +4215,7 @@
       <c r="L56" s="5"/>
       <c r="M56" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ищем управляющего кофейней: размещаем вакансию, приглашаем сильных кандидатов из других заведений, проводим собеседования и проверяем рекомендации. Результат: Управляющий выбран и готов выйти на обучение 25 января.</t>
+          <t xml:space="preserve">Ищем шефов, которые разработают меню выпечки и кофейную карту PECÀN и обучат команду. Результат: С шеф-пекарем и шеф-бариста заключены договоры на разработку меню.</t>
         </is>
       </c>
       <c r="N56" s="8"/>
@@ -4253,7 +4257,7 @@
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Подбор линейного персонала</t>
+          <t xml:space="preserve">Поиск управляющего</t>
         </is>
       </c>
       <c r="D57" s="3" t="inlineStr">
@@ -4263,10 +4267,10 @@
       </c>
       <c r="E57" s="3"/>
       <c r="F57" s="4">
-        <v>46391</v>
+        <v>46342</v>
       </c>
       <c r="G57" s="4">
-        <v>46416</v>
+        <v>46374</v>
       </c>
       <c r="H57" s="5">
         <f>G57-F57+1</f>
@@ -4281,7 +4285,7 @@
       <c r="L57" s="5"/>
       <c r="M57" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Набор команды: бариста, пекари, повара, кассиры, сотрудники зала и клининг. Вакансии, отбор анкет, собеседования, пробные смены. Результат: На каждую должность есть утверждённый кандидат с проверенными рекомендациями.</t>
+          <t xml:space="preserve">Ищем управляющего кофейней: размещаем вакансию, приглашаем сильных кандидатов из других заведений, проводим собеседования и проверяем рекомендации. Результат: Управляющий выбран и готов выйти на обучение 25 января.</t>
         </is>
       </c>
       <c r="N57" s="8"/>
@@ -4323,7 +4327,7 @@
       </c>
       <c r="C58" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Оформление сотрудников и медицинские книжки</t>
+          <t xml:space="preserve">Подбор линейного персонала</t>
         </is>
       </c>
       <c r="D58" s="3" t="inlineStr">
@@ -4333,10 +4337,10 @@
       </c>
       <c r="E58" s="3"/>
       <c r="F58" s="4">
-        <v>46412</v>
+        <v>46391</v>
       </c>
       <c r="G58" s="4">
-        <v>46423</v>
+        <v>46416</v>
       </c>
       <c r="H58" s="5">
         <f>G58-F58+1</f>
@@ -4351,7 +4355,7 @@
       <c r="L58" s="5"/>
       <c r="M58" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Официальное оформление сотрудников и прохождение медосмотра с получением медицинских книжек. Результат: Со всеми подписаны договоры, у каждого действующая медкнижка.</t>
+          <t xml:space="preserve">Набор команды: бариста, пекари, повара, кассиры, сотрудники зала и клининг. Вакансии, отбор анкет, собеседования, пробные смены. Результат: На каждую должность есть утверждённый кандидат с проверенными рекомендациями.</t>
         </is>
       </c>
       <c r="N58" s="8"/>
@@ -4391,9 +4395,9 @@
           <t xml:space="preserve">Команда</t>
         </is>
       </c>
-      <c r="C59" s="17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Штат укомплектован: 10–14 человек</t>
+      <c r="C59" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Оформление сотрудников и медицинские книжки</t>
         </is>
       </c>
       <c r="D59" s="3" t="inlineStr">
@@ -4403,10 +4407,10 @@
       </c>
       <c r="E59" s="3"/>
       <c r="F59" s="4">
-        <v>46416</v>
+        <v>46412</v>
       </c>
       <c r="G59" s="4">
-        <v>46416</v>
+        <v>46423</v>
       </c>
       <c r="H59" s="5">
         <f>G59-F59+1</f>
@@ -4417,15 +4421,11 @@
       <c r="J59" s="5" t="str">
         <f>IF(I59&gt;=1,"Готово",IF(G59&lt;TODAY(),"Просрочено",IF(F59&lt;=TODAY(),"В работе","В плане")))</f>
       </c>
-      <c r="K59" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">да</t>
-        </is>
-      </c>
+      <c r="K59" s="5"/>
       <c r="L59" s="5"/>
       <c r="M59" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Финальная проверка: все должности закрыты, люди подтвердили выход. Результат: Полный штат из 10–14 человек готов к обучению.</t>
+          <t xml:space="preserve">Официальное оформление сотрудников и прохождение медосмотра с получением медицинских книжек. Результат: Со всеми подписаны договоры, у каждого действующая медкнижка.</t>
         </is>
       </c>
       <c r="N59" s="8"/>
@@ -4462,12 +4462,12 @@
       </c>
       <c r="B60" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Меню и продукт</t>
-        </is>
-      </c>
-      <c r="C60" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Концепция меню</t>
+          <t xml:space="preserve">Команда</t>
+        </is>
+      </c>
+      <c r="C60" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Штат укомплектован: 10–14 человек</t>
         </is>
       </c>
       <c r="D60" s="3" t="inlineStr">
@@ -4475,16 +4475,12 @@
           <t xml:space="preserve">Команда PECÀN</t>
         </is>
       </c>
-      <c r="E60" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Шефы</t>
-        </is>
-      </c>
+      <c r="E60" s="3"/>
       <c r="F60" s="4">
-        <v>46335</v>
+        <v>46416</v>
       </c>
       <c r="G60" s="4">
-        <v>46353</v>
+        <v>46416</v>
       </c>
       <c r="H60" s="5">
         <f>G60-F60+1</f>
@@ -4495,11 +4491,15 @@
       <c r="J60" s="5" t="str">
         <f>IF(I60&gt;=1,"Готово",IF(G60&lt;TODAY(),"Просрочено",IF(F60&lt;=TODAY(),"В работе","В плане")))</f>
       </c>
-      <c r="K60" s="5"/>
+      <c r="K60" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">да</t>
+        </is>
+      </c>
       <c r="L60" s="5"/>
       <c r="M60" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Определяем, что будет в меню: категории, количество позиций, фирменные хиты, завтраки, сезонные предложения. Опираемся на ассортиментную матрицу и возможности оборудования. Результат: Утверждённая структура меню, по которой шефы пишут рецептуры.</t>
+          <t xml:space="preserve">Финальная проверка: все должности закрыты, люди подтвердили выход. Результат: Полный штат из 10–14 человек готов к обучению.</t>
         </is>
       </c>
       <c r="N60" s="8"/>
@@ -4541,20 +4541,24 @@
       </c>
       <c r="C61" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Рецептуры и технологические карты</t>
+          <t xml:space="preserve">Концепция меню</t>
         </is>
       </c>
       <c r="D61" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Шефы и персонал</t>
-        </is>
-      </c>
-      <c r="E61" s="3"/>
+          <t xml:space="preserve">Команда PECÀN</t>
+        </is>
+      </c>
+      <c r="E61" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Шефы</t>
+        </is>
+      </c>
       <c r="F61" s="4">
-        <v>46363</v>
+        <v>46335</v>
       </c>
       <c r="G61" s="4">
-        <v>46409</v>
+        <v>46353</v>
       </c>
       <c r="H61" s="5">
         <f>G61-F61+1</f>
@@ -4569,7 +4573,7 @@
       <c r="L61" s="5"/>
       <c r="M61" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Шефы разрабатывают рецепты и оформляют технологические карты: состав, граммовки, способ приготовления, себестоимость каждой позиции. Результат: На каждую позицию меню есть техкарта с себестоимостью и фото подачи.</t>
+          <t xml:space="preserve">Определяем, что будет в меню: категории, количество позиций, фирменные хиты, завтраки, сезонные предложения. Опираемся на ассортиментную матрицу и возможности оборудования. Результат: Утверждённая структура меню, по которой шефы пишут рецептуры.</t>
         </is>
       </c>
       <c r="N61" s="8"/>
@@ -4611,20 +4615,20 @@
       </c>
       <c r="C62" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Упаковка, печать меню, форма персонала</t>
+          <t xml:space="preserve">Рецептуры и технологические карты</t>
         </is>
       </c>
       <c r="D62" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Команда PECÀN</t>
+          <t xml:space="preserve">Шефы и персонал</t>
         </is>
       </c>
       <c r="E62" s="3"/>
       <c r="F62" s="4">
-        <v>46391</v>
+        <v>46363</v>
       </c>
       <c r="G62" s="4">
-        <v>46423</v>
+        <v>46409</v>
       </c>
       <c r="H62" s="5">
         <f>G62-F62+1</f>
@@ -4639,7 +4643,7 @@
       <c r="L62" s="5"/>
       <c r="M62" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Заказ стаканов, пакетов и коробок, печать меню и ценников, пошив формы. Всё по брендбуку, дизайн стаканов и крафтовых пакетов обновляется. Результат: Упаковка, меню и форма на объекте до технического открытия.</t>
+          <t xml:space="preserve">Шефы разрабатывают рецепты и оформляют технологические карты: состав, граммовки, способ приготовления, себестоимость каждой позиции. Результат: На каждую позицию меню есть техкарта с себестоимостью и фото подачи.</t>
         </is>
       </c>
       <c r="N62" s="8"/>
@@ -4681,7 +4685,7 @@
       </c>
       <c r="C63" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Поставщики сырья: отбор и договоры</t>
+          <t xml:space="preserve">Упаковка, печать меню, форма персонала</t>
         </is>
       </c>
       <c r="D63" s="3" t="inlineStr">
@@ -4691,7 +4695,7 @@
       </c>
       <c r="E63" s="3"/>
       <c r="F63" s="4">
-        <v>46398</v>
+        <v>46391</v>
       </c>
       <c r="G63" s="4">
         <v>46423</v>
@@ -4709,7 +4713,7 @@
       <c r="L63" s="5"/>
       <c r="M63" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Выбираем поставщиков кофе, молока, муки, масла и остальных продуктов: сравниваем качество, цены и условия доставки, заключаем договоры. Результат: На каждый ключевой продукт есть основной и запасной поставщик с договором.</t>
+          <t xml:space="preserve">Заказ стаканов, пакетов и коробок, печать меню и ценников, пошив формы. Всё по брендбуку, дизайн стаканов и крафтовых пакетов обновляется. Результат: Упаковка, меню и форма на объекте до технического открытия.</t>
         </is>
       </c>
       <c r="N63" s="8"/>
@@ -4751,20 +4755,20 @@
       </c>
       <c r="C64" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Проработки и дегустации на объекте</t>
+          <t xml:space="preserve">Поставщики сырья: отбор и договоры</t>
         </is>
       </c>
       <c r="D64" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Шефы и персонал</t>
+          <t xml:space="preserve">Команда PECÀN</t>
         </is>
       </c>
       <c r="E64" s="3"/>
       <c r="F64" s="4">
-        <v>46426</v>
+        <v>46398</v>
       </c>
       <c r="G64" s="4">
-        <v>46431</v>
+        <v>46423</v>
       </c>
       <c r="H64" s="5">
         <f>G64-F64+1</f>
@@ -4779,7 +4783,7 @@
       <c r="L64" s="5"/>
       <c r="M64" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Шефы готовят всё меню на нашем оборудовании, команда PECÀN пробует и даёт правки по вкусу, подаче и времени приготовления. Результат: Каждая позиция утверждена по вкусу и подаче, время отдачи укладывается в стандарт.</t>
+          <t xml:space="preserve">Выбираем поставщиков кофе, молока, муки, масла и остальных продуктов: сравниваем качество, цены и условия доставки, заключаем договоры. Результат: На каждый ключевой продукт есть основной и запасной поставщик с договором.</t>
         </is>
       </c>
       <c r="N64" s="8"/>
@@ -4816,25 +4820,25 @@
       </c>
       <c r="B65" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Автоматизация и IT</t>
+          <t xml:space="preserve">Меню и продукт</t>
         </is>
       </c>
       <c r="C65" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Закупка касс, принтеров, лицензий iiko</t>
+          <t xml:space="preserve">Проработки и дегустации на объекте</t>
         </is>
       </c>
       <c r="D65" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Команда PECÀN</t>
+          <t xml:space="preserve">Шефы и персонал</t>
         </is>
       </c>
       <c r="E65" s="3"/>
       <c r="F65" s="4">
-        <v>46398</v>
+        <v>46426</v>
       </c>
       <c r="G65" s="4">
-        <v>46409</v>
+        <v>46431</v>
       </c>
       <c r="H65" s="5">
         <f>G65-F65+1</f>
@@ -4849,7 +4853,7 @@
       <c r="L65" s="5"/>
       <c r="M65" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Покупка кассовых моноблоков, принтеров чеков и лицензий iiko. Результат: Оборудование и лицензии на руках, можно начинать настройку.</t>
+          <t xml:space="preserve">Шефы готовят всё меню на нашем оборудовании, команда PECÀN пробует и даёт правки по вкусу, подаче и времени приготовления. Результат: Каждая позиция утверждена по вкусу и подаче, время отдачи укладывается в стандарт.</t>
         </is>
       </c>
       <c r="N65" s="8"/>
@@ -4891,7 +4895,7 @@
       </c>
       <c r="C66" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Настройка iiko: номенклатура, склады, техкарты</t>
+          <t xml:space="preserve">Закупка касс, принтеров, лицензий iiko</t>
         </is>
       </c>
       <c r="D66" s="3" t="inlineStr">
@@ -4901,10 +4905,10 @@
       </c>
       <c r="E66" s="3"/>
       <c r="F66" s="4">
-        <v>46412</v>
+        <v>46398</v>
       </c>
       <c r="G66" s="4">
-        <v>46430</v>
+        <v>46409</v>
       </c>
       <c r="H66" s="5">
         <f>G66-F66+1</f>
@@ -4919,7 +4923,7 @@
       <c r="L66" s="5"/>
       <c r="M66" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Настраиваем систему учёта: заносим меню, склады, техкарты шефов и правила списания продуктов. Результат: Каждая продажа автоматически списывает продукты со склада, остатки видны в системе.</t>
+          <t xml:space="preserve">Покупка кассовых моноблоков, принтеров чеков и лицензий iiko. Результат: Оборудование и лицензии на руках, можно начинать настройку.</t>
         </is>
       </c>
       <c r="N66" s="8"/>
@@ -4961,7 +4965,7 @@
       </c>
       <c r="C67" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Бонусная программа лояльности</t>
+          <t xml:space="preserve">Настройка iiko: номенклатура, склады, техкарты</t>
         </is>
       </c>
       <c r="D67" s="3" t="inlineStr">
@@ -4971,7 +4975,7 @@
       </c>
       <c r="E67" s="3"/>
       <c r="F67" s="4">
-        <v>46419</v>
+        <v>46412</v>
       </c>
       <c r="G67" s="4">
         <v>46430</v>
@@ -4989,7 +4993,7 @@
       <c r="L67" s="5"/>
       <c r="M67" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Настраиваем бонусную программу для гостей и связываем её с кассой, обучаем кассиров. Результат: Гость регистрируется за минуту, бонусы начисляются и списываются на кассе.</t>
+          <t xml:space="preserve">Настраиваем систему учёта: заносим меню, склады, техкарты шефов и правила списания продуктов. Результат: Каждая продажа автоматически списывает продукты со склада, остатки видны в системе.</t>
         </is>
       </c>
       <c r="N67" s="8"/>
@@ -5031,7 +5035,7 @@
       </c>
       <c r="C68" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kaspi Pay, Webkassa, кассовая зона</t>
+          <t xml:space="preserve">Бонусная программа лояльности</t>
         </is>
       </c>
       <c r="D68" s="3" t="inlineStr">
@@ -5059,7 +5063,7 @@
       <c r="L68" s="5"/>
       <c r="M68" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Подключаем оплату через Kaspi и картой, онлайн-кассу Webkassa, принтеры на баре и кухне. Результат: Тестовая продажа проходит целиком: заказ, оплата, чек, заказ на кухне.</t>
+          <t xml:space="preserve">Настраиваем бонусную программу для гостей и связываем её с кассой, обучаем кассиров. Результат: Гость регистрируется за минуту, бонусы начисляются и списываются на кассе.</t>
         </is>
       </c>
       <c r="N68" s="8"/>
@@ -5101,7 +5105,7 @@
       </c>
       <c r="C69" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Дашборд для владельцев</t>
+          <t xml:space="preserve">Kaspi Pay, Webkassa, кассовая зона</t>
         </is>
       </c>
       <c r="D69" s="3" t="inlineStr">
@@ -5111,10 +5115,10 @@
       </c>
       <c r="E69" s="3"/>
       <c r="F69" s="4">
-        <v>46426</v>
+        <v>46419</v>
       </c>
       <c r="G69" s="4">
-        <v>46437</v>
+        <v>46430</v>
       </c>
       <c r="H69" s="5">
         <f>G69-F69+1</f>
@@ -5129,7 +5133,7 @@
       <c r="L69" s="5"/>
       <c r="M69" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Настраиваем отчёты, которые владельцы видят с телефона: выручка, средний чек, количество гостей, остатки. Результат: Вы открываете приложение и видите выручку за сегодня в реальном времени.</t>
+          <t xml:space="preserve">Подключаем оплату через Kaspi и картой, онлайн-кассу Webkassa, принтеры на баре и кухне. Результат: Тестовая продажа проходит целиком: заказ, оплата, чек, заказ на кухне.</t>
         </is>
       </c>
       <c r="N69" s="8"/>
@@ -5171,7 +5175,7 @@
       </c>
       <c r="C70" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Заявки в Wolt, Yandex Eats, Glovo, Choco</t>
+          <t xml:space="preserve">Дашборд для владельцев</t>
         </is>
       </c>
       <c r="D70" s="3" t="inlineStr">
@@ -5184,7 +5188,7 @@
         <v>46426</v>
       </c>
       <c r="G70" s="4">
-        <v>46444</v>
+        <v>46437</v>
       </c>
       <c r="H70" s="5">
         <f>G70-F70+1</f>
@@ -5199,7 +5203,7 @@
       <c r="L70" s="5"/>
       <c r="M70" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Готовим меню доставки и подаём заявки на подключение. Решение о подключении принимают сами сервисы. Результат: Заявки поданы во все четыре сервиса, меню и фото готовы.</t>
+          <t xml:space="preserve">Настраиваем отчёты, которые владельцы видят с телефона: выручка, средний чек, количество гостей, остатки. Результат: Вы открываете приложение и видите выручку за сегодня в реальном времени.</t>
         </is>
       </c>
       <c r="N70" s="8"/>
@@ -5236,12 +5240,12 @@
       </c>
       <c r="B71" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Стандарты и обучение</t>
+          <t xml:space="preserve">Автоматизация и IT</t>
         </is>
       </c>
       <c r="C71" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Service Book, должностные инструкции, чек-листы, ХАССП</t>
+          <t xml:space="preserve">Заявки в Wolt, Yandex Eats, Glovo, Choco</t>
         </is>
       </c>
       <c r="D71" s="3" t="inlineStr">
@@ -5251,10 +5255,10 @@
       </c>
       <c r="E71" s="3"/>
       <c r="F71" s="4">
-        <v>46342</v>
+        <v>46426</v>
       </c>
       <c r="G71" s="4">
-        <v>46374</v>
+        <v>46444</v>
       </c>
       <c r="H71" s="5">
         <f>G71-F71+1</f>
@@ -5269,7 +5273,7 @@
       <c r="L71" s="5"/>
       <c r="M71" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Пишем правила работы кофейни: как встречать гостя и готовить заказ, кто за что отвечает, что делать при открытии и закрытии смены, как соблюдать санитарные нормы. Результат: Комплект документов, по которым новый сотрудник понимает свою работу с первого дня.</t>
+          <t xml:space="preserve">Готовим меню доставки и подаём заявки на подключение. Решение о подключении принимают сами сервисы. Результат: Заявки поданы во все четыре сервиса, меню и фото готовы.</t>
         </is>
       </c>
       <c r="N71" s="8"/>
@@ -5311,7 +5315,7 @@
       </c>
       <c r="C72" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Обучение управляющего</t>
+          <t xml:space="preserve">Service Book, должностные инструкции, чек-листы, ХАССП</t>
         </is>
       </c>
       <c r="D72" s="3" t="inlineStr">
@@ -5321,10 +5325,10 @@
       </c>
       <c r="E72" s="3"/>
       <c r="F72" s="4">
-        <v>46412</v>
+        <v>46342</v>
       </c>
       <c r="G72" s="4">
-        <v>46423</v>
+        <v>46374</v>
       </c>
       <c r="H72" s="5">
         <f>G72-F72+1</f>
@@ -5339,7 +5343,7 @@
       <c r="L72" s="5"/>
       <c r="M72" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Учим управляющего вести кофейню: графики смен, заказ продуктов, себестоимость, инвентаризация, работа с отзывами и жалобами. Результат: Управляющий самостоятельно составляет график, делает заказ поставщикам и читает отчёты.</t>
+          <t xml:space="preserve">Пишем правила работы кофейни: как встречать гостя и готовить заказ, кто за что отвечает, что делать при открытии и закрытии смены, как соблюдать санитарные нормы. Результат: Комплект документов, по которым новый сотрудник понимает свою работу с первого дня.</t>
         </is>
       </c>
       <c r="N72" s="8"/>
@@ -5381,7 +5385,7 @@
       </c>
       <c r="C73" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Договоры ЖКХ, вывоз отходов, уведомление о начале деятельности</t>
+          <t xml:space="preserve">Обучение управляющего</t>
         </is>
       </c>
       <c r="D73" s="3" t="inlineStr">
@@ -5394,7 +5398,7 @@
         <v>46412</v>
       </c>
       <c r="G73" s="4">
-        <v>46430</v>
+        <v>46423</v>
       </c>
       <c r="H73" s="5">
         <f>G73-F73+1</f>
@@ -5409,7 +5413,7 @@
       <c r="L73" s="5"/>
       <c r="M73" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Договоры на электричество, воду, вывоз мусора и дезинсекцию, уведомление о начале деятельности. Результат: Все договоры подписаны, уведомление подано, можно легально работать.</t>
+          <t xml:space="preserve">Учим управляющего вести кофейню: графики смен, заказ продуктов, себестоимость, инвентаризация, работа с отзывами и жалобами. Результат: Управляющий самостоятельно составляет график, делает заказ поставщикам и читает отчёты.</t>
         </is>
       </c>
       <c r="N73" s="8"/>
@@ -5451,7 +5455,7 @@
       </c>
       <c r="C74" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Академия PECÀN: бариста, пекарня, кухня, сервис</t>
+          <t xml:space="preserve">Договоры ЖКХ, вывоз отходов, уведомление о начале деятельности</t>
         </is>
       </c>
       <c r="D74" s="3" t="inlineStr">
@@ -5459,16 +5463,12 @@
           <t xml:space="preserve">Команда PECÀN</t>
         </is>
       </c>
-      <c r="E74" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Персонал кофейни</t>
-        </is>
-      </c>
+      <c r="E74" s="3"/>
       <c r="F74" s="4">
-        <v>46426</v>
+        <v>46412</v>
       </c>
       <c r="G74" s="4">
-        <v>46431</v>
+        <v>46430</v>
       </c>
       <c r="H74" s="5">
         <f>G74-F74+1</f>
@@ -5480,14 +5480,10 @@
         <f>IF(I74&gt;=1,"Готово",IF(G74&lt;TODAY(),"Просрочено",IF(F74&lt;=TODAY(),"В работе","В плане")))</f>
       </c>
       <c r="K74" s="5"/>
-      <c r="L74" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">да</t>
-        </is>
-      </c>
+      <c r="L74" s="5"/>
       <c r="M74" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Неделя обучения всей команды: бариста тренируют кофе и скорость, пекари и повара работают по техкартам, зал и касса учат меню и стандарты общения с гостем. Результат: Каждый сотрудник знает меню и свои действия на смене, готов к аттестации.</t>
+          <t xml:space="preserve">Договоры на электричество, воду, вывоз мусора и дезинсекцию, уведомление о начале деятельности. Результат: Все договоры подписаны, уведомление подано, можно легально работать.</t>
         </is>
       </c>
       <c r="N74" s="8"/>
@@ -5527,9 +5523,9 @@
           <t xml:space="preserve">Стандарты и обучение</t>
         </is>
       </c>
-      <c r="C75" s="17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Аттестация команды</t>
+      <c r="C75" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Академия PECÀN: бариста, пекарня, кухня, сервис</t>
         </is>
       </c>
       <c r="D75" s="3" t="inlineStr">
@@ -5537,9 +5533,13 @@
           <t xml:space="preserve">Команда PECÀN</t>
         </is>
       </c>
-      <c r="E75" s="3"/>
+      <c r="E75" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Персонал кофейни</t>
+        </is>
+      </c>
       <c r="F75" s="4">
-        <v>46431</v>
+        <v>46426</v>
       </c>
       <c r="G75" s="4">
         <v>46431</v>
@@ -5553,19 +5553,15 @@
       <c r="J75" s="5" t="str">
         <f>IF(I75&gt;=1,"Готово",IF(G75&lt;TODAY(),"Просрочено",IF(F75&lt;=TODAY(),"В работе","В плане")))</f>
       </c>
-      <c r="K75" s="5" t="inlineStr">
+      <c r="K75" s="5"/>
+      <c r="L75" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">да</t>
         </is>
       </c>
-      <c r="L75" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">да</t>
-        </is>
-      </c>
       <c r="M75" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Экзамен для каждого сотрудника: теория по меню и стандартам плюс практика на рабочем месте. Результат: К смене допущены только те, кто сдал аттестацию.</t>
+          <t xml:space="preserve">Неделя обучения всей команды: бариста тренируют кофе и скорость, пекари и повара работают по техкартам, зал и касса учат меню и стандарты общения с гостем. Результат: Каждый сотрудник знает меню и свои действия на смене, готов к аттестации.</t>
         </is>
       </c>
       <c r="N75" s="8"/>
@@ -5602,12 +5598,12 @@
       </c>
       <c r="B76" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Маркетинг запуска</t>
-        </is>
-      </c>
-      <c r="C76" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Медиаплан запуска</t>
+          <t xml:space="preserve">Стандарты и обучение</t>
+        </is>
+      </c>
+      <c r="C76" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Аттестация команды</t>
         </is>
       </c>
       <c r="D76" s="3" t="inlineStr">
@@ -5617,10 +5613,10 @@
       </c>
       <c r="E76" s="3"/>
       <c r="F76" s="4">
-        <v>46321</v>
+        <v>46431</v>
       </c>
       <c r="G76" s="4">
-        <v>46339</v>
+        <v>46431</v>
       </c>
       <c r="H76" s="5">
         <f>G76-F76+1</f>
@@ -5631,11 +5627,19 @@
       <c r="J76" s="5" t="str">
         <f>IF(I76&gt;=1,"Готово",IF(G76&lt;TODAY(),"Просрочено",IF(F76&lt;=TODAY(),"В работе","В плане")))</f>
       </c>
-      <c r="K76" s="5"/>
-      <c r="L76" s="5"/>
+      <c r="K76" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">да</t>
+        </is>
+      </c>
+      <c r="L76" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">да</t>
+        </is>
+      </c>
       <c r="M76" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">План продвижения: что, где и когда публикуем до и после открытия, какие активности проводим, какой бюджет на рекламу нужен. Результат: Календарь публикаций и активностей с бюджетом по неделям.</t>
+          <t xml:space="preserve">Экзамен для каждого сотрудника: теория по меню и стандартам плюс практика на рабочем месте. Результат: К смене допущены только те, кто сдал аттестацию.</t>
         </is>
       </c>
       <c r="N76" s="8"/>
@@ -5677,7 +5681,7 @@
       </c>
       <c r="C77" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Instagram: прогрев до открытия</t>
+          <t xml:space="preserve">Медиаплан запуска</t>
         </is>
       </c>
       <c r="D77" s="3" t="inlineStr">
@@ -5687,10 +5691,10 @@
       </c>
       <c r="E77" s="3"/>
       <c r="F77" s="4">
-        <v>46391</v>
+        <v>46321</v>
       </c>
       <c r="G77" s="4">
-        <v>46459</v>
+        <v>46339</v>
       </c>
       <c r="H77" s="5">
         <f>G77-F77+1</f>
@@ -5705,7 +5709,7 @@
       <c r="L77" s="5"/>
       <c r="M77" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ведём аккаунт до открытия: показываем ремонт, команду, пробы меню, собираем аудиторию района. Результат: К открытию у аккаунта есть живые подписчики из района, которые ждут запуска.</t>
+          <t xml:space="preserve">План продвижения: что, где и когда публикуем до и после открытия, какие активности проводим, какой бюджет на рекламу нужен. Результат: Календарь публикаций и активностей с бюджетом по неделям.</t>
         </is>
       </c>
       <c r="N77" s="8"/>
@@ -5747,7 +5751,7 @@
       </c>
       <c r="C78" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Карточки в 2ГИС, Яндекс и Google</t>
+          <t xml:space="preserve">Instagram: прогрев до открытия</t>
         </is>
       </c>
       <c r="D78" s="3" t="inlineStr">
@@ -5757,10 +5761,10 @@
       </c>
       <c r="E78" s="3"/>
       <c r="F78" s="4">
-        <v>46419</v>
+        <v>46391</v>
       </c>
       <c r="G78" s="4">
-        <v>46430</v>
+        <v>46459</v>
       </c>
       <c r="H78" s="5">
         <f>G78-F78+1</f>
@@ -5775,7 +5779,7 @@
       <c r="L78" s="5"/>
       <c r="M78" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Создаём и оформляем карточки заведения на картах: адрес, часы работы, фото, меню. Результат: PECÀN находится в поиске на картах, информация и фото актуальны.</t>
+          <t xml:space="preserve">Ведём аккаунт до открытия: показываем ремонт, команду, пробы меню, собираем аудиторию района. Результат: К открытию у аккаунта есть живые подписчики из района, которые ждут запуска.</t>
         </is>
       </c>
       <c r="N78" s="8"/>
@@ -5817,7 +5821,7 @@
       </c>
       <c r="C79" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Подготовка торжественного открытия</t>
+          <t xml:space="preserve">Карточки в 2ГИС, Яндекс и Google</t>
         </is>
       </c>
       <c r="D79" s="3" t="inlineStr">
@@ -5827,10 +5831,10 @@
       </c>
       <c r="E79" s="3"/>
       <c r="F79" s="4">
-        <v>46433</v>
+        <v>46419</v>
       </c>
       <c r="G79" s="4">
-        <v>46458</v>
+        <v>46430</v>
       </c>
       <c r="H79" s="5">
         <f>G79-F79+1</f>
@@ -5845,7 +5849,7 @@
       <c r="L79" s="5"/>
       <c r="M79" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Готовим торжественное открытие: программа дня, приглашения блогерам и гостям, подарки, фото и видеосъёмка. Результат: Сценарий утверждён, гости приглашены, всё закуплено за день до события.</t>
+          <t xml:space="preserve">Создаём и оформляем карточки заведения на картах: адрес, часы работы, фото, меню. Результат: PECÀN находится в поиске на картах, информация и фото актуальны.</t>
         </is>
       </c>
       <c r="N79" s="8"/>
@@ -5882,12 +5886,12 @@
       </c>
       <c r="B80" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Запуск</t>
+          <t xml:space="preserve">Маркетинг запуска</t>
         </is>
       </c>
       <c r="C80" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Первый закуп продуктов и расходников</t>
+          <t xml:space="preserve">Подготовка торжественного открытия</t>
         </is>
       </c>
       <c r="D80" s="3" t="inlineStr">
@@ -5897,10 +5901,10 @@
       </c>
       <c r="E80" s="3"/>
       <c r="F80" s="4">
-        <v>46428</v>
+        <v>46433</v>
       </c>
       <c r="G80" s="4">
-        <v>46432</v>
+        <v>46458</v>
       </c>
       <c r="H80" s="5">
         <f>G80-F80+1</f>
@@ -5915,7 +5919,7 @@
       <c r="L80" s="5"/>
       <c r="M80" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Первая закупка продуктов, кофе, молока, упаковки и расходников под стартовое меню. Результат: Склад заполнен на первую неделю работы.</t>
+          <t xml:space="preserve">Готовим торжественное открытие: программа дня, приглашения блогерам и гостям, подарки, фото и видеосъёмка. Результат: Сценарий утверждён, гости приглашены, всё закуплено за день до события.</t>
         </is>
       </c>
       <c r="N80" s="8"/>
@@ -5955,9 +5959,9 @@
           <t xml:space="preserve">Запуск</t>
         </is>
       </c>
-      <c r="C81" s="17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Техническое открытие</t>
+      <c r="C81" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Первый закуп продуктов и расходников</t>
         </is>
       </c>
       <c r="D81" s="3" t="inlineStr">
@@ -5965,16 +5969,12 @@
           <t xml:space="preserve">Команда PECÀN</t>
         </is>
       </c>
-      <c r="E81" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Все участники</t>
-        </is>
-      </c>
+      <c r="E81" s="3"/>
       <c r="F81" s="4">
-        <v>46433</v>
+        <v>46428</v>
       </c>
       <c r="G81" s="4">
-        <v>46433</v>
+        <v>46432</v>
       </c>
       <c r="H81" s="5">
         <f>G81-F81+1</f>
@@ -5985,19 +5985,11 @@
       <c r="J81" s="5" t="str">
         <f>IF(I81&gt;=1,"Готово",IF(G81&lt;TODAY(),"Просрочено",IF(F81&lt;=TODAY(),"В работе","В плане")))</f>
       </c>
-      <c r="K81" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">да</t>
-        </is>
-      </c>
-      <c r="L81" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">да</t>
-        </is>
-      </c>
+      <c r="K81" s="5"/>
+      <c r="L81" s="5"/>
       <c r="M81" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Первый рабочий день без рекламы и вывески о запуске. Принимаем первых гостей и проверяем все процессы в реальной работе. Результат: Кофейня открыла двери и отработала полную смену.</t>
+          <t xml:space="preserve">Первая закупка продуктов, кофе, молока, упаковки и расходников под стартовое меню. Результат: Склад заполнен на первую неделю работы.</t>
         </is>
       </c>
       <c r="N81" s="8"/>
@@ -6037,9 +6029,9 @@
           <t xml:space="preserve">Запуск</t>
         </is>
       </c>
-      <c r="C82" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Тестовая эксплуатация, 10 дней</t>
+      <c r="C82" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Техническое открытие</t>
         </is>
       </c>
       <c r="D82" s="3" t="inlineStr">
@@ -6049,14 +6041,14 @@
       </c>
       <c r="E82" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Персонал кофейни</t>
+          <t xml:space="preserve">Все участники</t>
         </is>
       </c>
       <c r="F82" s="4">
         <v>46433</v>
       </c>
       <c r="G82" s="4">
-        <v>46442</v>
+        <v>46433</v>
       </c>
       <c r="H82" s="5">
         <f>G82-F82+1</f>
@@ -6067,7 +6059,11 @@
       <c r="J82" s="5" t="str">
         <f>IF(I82&gt;=1,"Готово",IF(G82&lt;TODAY(),"Просрочено",IF(F82&lt;=TODAY(),"В работе","В плане")))</f>
       </c>
-      <c r="K82" s="5"/>
+      <c r="K82" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">да</t>
+        </is>
+      </c>
       <c r="L82" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">да</t>
@@ -6075,7 +6071,7 @@
       </c>
       <c r="M82" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Десять дней работаем в тихом режиме: закрытая фокус-группа, друзья и соседи. Замеряем скорость отдачи, собираем отзывы, находим узкие места. Результат: Список проблем найден и устранён, заказ отдаётся за стандартное время даже в пик.</t>
+          <t xml:space="preserve">Первый рабочий день без рекламы и вывески о запуске. Принимаем первых гостей и проверяем все процессы в реальной работе. Результат: Кофейня открыла двери и отработала полную смену.</t>
         </is>
       </c>
       <c r="N82" s="8"/>
@@ -6117,20 +6113,24 @@
       </c>
       <c r="C83" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Работа в мягком режиме, доводка процессов</t>
+          <t xml:space="preserve">Тестовая эксплуатация, 10 дней</t>
         </is>
       </c>
       <c r="D83" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Шефы и персонал</t>
-        </is>
-      </c>
-      <c r="E83" s="3"/>
+          <t xml:space="preserve">Команда PECÀN</t>
+        </is>
+      </c>
+      <c r="E83" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Персонал кофейни</t>
+        </is>
+      </c>
       <c r="F83" s="4">
-        <v>46443</v>
+        <v>46433</v>
       </c>
       <c r="G83" s="4">
-        <v>46458</v>
+        <v>46442</v>
       </c>
       <c r="H83" s="5">
         <f>G83-F83+1</f>
@@ -6142,10 +6142,14 @@
         <f>IF(I83&gt;=1,"Готово",IF(G83&lt;TODAY(),"Просрочено",IF(F83&lt;=TODAY(),"В работе","В плане")))</f>
       </c>
       <c r="K83" s="5"/>
-      <c r="L83" s="5"/>
+      <c r="L83" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">да</t>
+        </is>
+      </c>
       <c r="M83" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Работаем для всех, но без громкой рекламы. Команда набирает скорость, докручиваем меню и процессы по отзывам гостей. Результат: Команда уверенно проходит пиковые часы, отзывы на картах положительные.</t>
+          <t xml:space="preserve">Десять дней работаем в тихом режиме: закрытая фокус-группа, друзья и соседи. Замеряем скорость отдачи, собираем отзывы, находим узкие места. Результат: Список проблем найден и устранён, заказ отдаётся за стандартное время даже в пик.</t>
         </is>
       </c>
       <c r="N83" s="8"/>
@@ -6185,26 +6189,22 @@
           <t xml:space="preserve">Запуск</t>
         </is>
       </c>
-      <c r="C84" s="17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Торжественное открытие</t>
+      <c r="C84" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Работа в мягком режиме, доводка процессов</t>
         </is>
       </c>
       <c r="D84" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Команда PECÀN</t>
-        </is>
-      </c>
-      <c r="E84" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Все участники</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Шефы и персонал</t>
+        </is>
+      </c>
+      <c r="E84" s="3"/>
       <c r="F84" s="4">
-        <v>46459</v>
+        <v>46443</v>
       </c>
       <c r="G84" s="4">
-        <v>46459</v>
+        <v>46458</v>
       </c>
       <c r="H84" s="5">
         <f>G84-F84+1</f>
@@ -6215,19 +6215,11 @@
       <c r="J84" s="5" t="str">
         <f>IF(I84&gt;=1,"Готово",IF(G84&lt;TODAY(),"Просрочено",IF(F84&lt;=TODAY(),"В работе","В плане")))</f>
       </c>
-      <c r="K84" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">да</t>
-        </is>
-      </c>
-      <c r="L84" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">да</t>
-        </is>
-      </c>
+      <c r="K84" s="5"/>
+      <c r="L84" s="5"/>
       <c r="M84" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Официальное открытие PECÀN с гостями, блогерами и праздничной программой. Результат: Праздник прошёл, о PECÀN узнал район, первые публикации вышли.</t>
+          <t xml:space="preserve">Работаем для всех, но без громкой рекламы. Команда набирает скорость, докручиваем меню и процессы по отзывам гостей. Результат: Команда уверенно проходит пиковые часы, отзывы на картах положительные.</t>
         </is>
       </c>
       <c r="N84" s="8"/>
@@ -6267,9 +6259,9 @@
           <t xml:space="preserve">Запуск</t>
         </is>
       </c>
-      <c r="C85" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Итоговый аудит и акт, передача кофейни владельцам</t>
+      <c r="C85" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Торжественное открытие</t>
         </is>
       </c>
       <c r="D85" s="3" t="inlineStr">
@@ -6277,12 +6269,16 @@
           <t xml:space="preserve">Команда PECÀN</t>
         </is>
       </c>
-      <c r="E85" s="3"/>
+      <c r="E85" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Все участники</t>
+        </is>
+      </c>
       <c r="F85" s="4">
-        <v>46461</v>
+        <v>46459</v>
       </c>
       <c r="G85" s="4">
-        <v>46465</v>
+        <v>46459</v>
       </c>
       <c r="H85" s="5">
         <f>G85-F85+1</f>
@@ -6293,11 +6289,19 @@
       <c r="J85" s="5" t="str">
         <f>IF(I85&gt;=1,"Готово",IF(G85&lt;TODAY(),"Просрочено",IF(F85&lt;=TODAY(),"В работе","В плане")))</f>
       </c>
-      <c r="K85" s="5"/>
-      <c r="L85" s="5"/>
+      <c r="K85" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">да</t>
+        </is>
+      </c>
+      <c r="L85" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">да</t>
+        </is>
+      </c>
       <c r="M85" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Проверяем работу кофейни после открытия, передаём все документы, доступы и контакты, подписываем итоговый акт. Результат: Кофейня работает самостоятельно, у владельцев есть все документы и доступы.</t>
+          <t xml:space="preserve">Официальное открытие PECÀN с гостями, блогерами и праздничной программой. Результат: Праздник прошёл, о PECÀN узнал район, первые публикации вышли.</t>
         </is>
       </c>
       <c r="N85" s="8"/>
@@ -6328,9 +6332,79 @@
       <c r="AM85" s="8"/>
       <c r="AN85" s="8"/>
     </row>
+    <row r="86">
+      <c r="A86" s="5">
+        <v>82</v>
+      </c>
+      <c r="B86" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Запуск</t>
+        </is>
+      </c>
+      <c r="C86" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Итоговый аудит и акт, передача кофейни владельцам</t>
+        </is>
+      </c>
+      <c r="D86" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Команда PECÀN</t>
+        </is>
+      </c>
+      <c r="E86" s="3"/>
+      <c r="F86" s="4">
+        <v>46461</v>
+      </c>
+      <c r="G86" s="4">
+        <v>46465</v>
+      </c>
+      <c r="H86" s="5">
+        <f>G86-F86+1</f>
+      </c>
+      <c r="I86" s="6">
+        <v>0</v>
+      </c>
+      <c r="J86" s="5" t="str">
+        <f>IF(I86&gt;=1,"Готово",IF(G86&lt;TODAY(),"Просрочено",IF(F86&lt;=TODAY(),"В работе","В плане")))</f>
+      </c>
+      <c r="K86" s="5"/>
+      <c r="L86" s="5"/>
+      <c r="M86" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Проверяем работу кофейни после открытия, передаём все документы, доступы и контакты, подписываем итоговый акт. Результат: Кофейня работает самостоятельно, у владельцев есть все документы и доступы.</t>
+        </is>
+      </c>
+      <c r="N86" s="8"/>
+      <c r="O86" s="8"/>
+      <c r="P86" s="8"/>
+      <c r="Q86" s="8"/>
+      <c r="R86" s="8"/>
+      <c r="S86" s="8"/>
+      <c r="T86" s="8"/>
+      <c r="U86" s="8"/>
+      <c r="V86" s="8"/>
+      <c r="W86" s="8"/>
+      <c r="X86" s="8"/>
+      <c r="Y86" s="8"/>
+      <c r="Z86" s="8"/>
+      <c r="AA86" s="8"/>
+      <c r="AB86" s="8"/>
+      <c r="AC86" s="8"/>
+      <c r="AD86" s="8"/>
+      <c r="AE86" s="8"/>
+      <c r="AF86" s="8"/>
+      <c r="AG86" s="8"/>
+      <c r="AH86" s="8"/>
+      <c r="AI86" s="8"/>
+      <c r="AJ86" s="8"/>
+      <c r="AK86" s="8"/>
+      <c r="AL86" s="8"/>
+      <c r="AM86" s="8"/>
+      <c r="AN86" s="8"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:M85"/>
-  <conditionalFormatting sqref="N5:AN85">
+  <autoFilter ref="A4:M86"/>
+  <conditionalFormatting sqref="N5:AN86">
     <cfRule type="expression" dxfId="0" priority="1">
       <formula>AND($D5="Команда PECÀN",$F5&lt;=N$4+6,$G5&gt;=N$4)</formula>
     </cfRule>
@@ -6350,7 +6424,7 @@
       <formula>AND($D5="Шефы и персонал",$F5&lt;=N$4+6,$G5&gt;=N$4)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J5:J85">
+  <conditionalFormatting sqref="J5:J86">
     <cfRule type="cellIs" dxfId="6" priority="7" operator="equal">
       <formula>"Просрочено"</formula>
     </cfRule>
@@ -6359,7 +6433,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" sqref="D5:D125">
+    <dataValidation type="list" allowBlank="1" sqref="D5:D126">
       <formula1>"Команда PECÀN,Дизайн-студия,Строители,Поставщики и логистика,Шефы и персонал"</formula1>
     </dataValidation>
   </dataValidations>
@@ -6573,7 +6647,7 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Раздел ТХ и инженерные ТЗ сданы</t>
+          <t xml:space="preserve">Раздел ТХ и задание на инженерные сети сданы</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
@@ -6588,7 +6662,7 @@
       </c>
       <c r="G10" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Передача готового раздела ТХ и инженерных ТЗ. С этого момента строители могут выходить на объект.</t>
+          <t xml:space="preserve">Передача готового раздела ТХ и задания на инженерные сети. С этого момента строители могут выходить на объект и делать рабочие схемы.</t>
         </is>
       </c>
     </row>
@@ -6978,7 +7052,7 @@
         <is>
           <t xml:space="preserve">• Ведёт проект целиком: график, решения, согласования, бюджет
 • Аналитика локации, финансовая модель, маркетинговая стратегия
-• Технологический проект, инженерные ТЗ, технологический надзор
+• Технологический проект, задание на инженерные сети, технологический надзор
 • Выбор дизайн-студии и строительной бригады, договоры с подрядчиками
 • Спецификации, выездная сессия в Китае, оплата оборудования и логистики
 • Юрлицо, счёт, договоры с ЖКХ и поставщиками сырья
@@ -7005,13 +7079,13 @@
         <is>
           <t xml:space="preserve">• Планировочное решение и концепция интерьера
 • 3D-визуализации, сверка с технологическим зонированием
-• Рабочие чертежи, ведомости отделки, мебели и света, смета
+• Рабочие чертежи, план освещения и розеток, ведомости, смета
 • Авторский надзор за отделкой и декором
 • Эскиз фасадной вывески</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="86" customHeight="1">
+    <row r="7" ht="102" customHeight="1">
       <c r="A7" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">Строители</t>
@@ -7028,6 +7102,7 @@
       <c r="D7" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">• Черновые работы и перегородки по проекту
+• Рабочие схемы сетей с расчётами
 • Электрика 380 В, вода, канализация, трапы, жироуловитель
 • Вентиляция и кондиционирование
 • Чистовая отделка, свет, сантехника

</xml_diff>

<commit_message>
Plan update 2026-10-10: traffic estimate and competitor analysis closed
</commit_message>
<xml_diff>
--- a/pecan-plan.xlsx
+++ b/pecan-plan.xlsx
@@ -286,7 +286,7 @@
     <row r="2">
       <c r="A2" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Астана, пр. Тұран, 52/4 · ведёт команда PECÀN · состояние на 5 окт 2026 · даты, проценты и ответственных можно менять, полосы справа пересчитаются сами</t>
+          <t xml:space="preserve">Астана, пр. Тұран, 52/4 · ведёт команда PECÀN · состояние на 10 окт 2026 · даты, проценты и ответственных можно менять, полосы справа пересчитаются сами</t>
         </is>
       </c>
     </row>
@@ -752,7 +752,7 @@
         <f>G9-F9+1</f>
       </c>
       <c r="I9" s="6">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="J9" s="5" t="str">
         <f>IF(I9&gt;=1,"Готово",IF(G9&lt;TODAY(),"Просрочено",IF(F9&lt;=TODAY(),"В работе","В плане")))</f>
@@ -803,7 +803,7 @@
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Замер проходящего и проезжающего трафика у входа</t>
+          <t xml:space="preserve">Оценка трафика у входа: расчётная модель</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
@@ -816,13 +816,13 @@
         <v>46293</v>
       </c>
       <c r="G10" s="4">
-        <v>46306</v>
+        <v>46305</v>
       </c>
       <c r="H10" s="5">
         <f>G10-F10+1</f>
       </c>
       <c r="I10" s="6">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="J10" s="5" t="str">
         <f>IF(I10&gt;=1,"Готово",IF(G10&lt;TODAY(),"Просрочено",IF(F10&lt;=TODAY(),"В работе","В плане")))</f>
@@ -831,7 +831,7 @@
       <c r="L10" s="5"/>
       <c r="M10" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Вход в кофейню выходит на внутреннюю аллею, поэтому считаем именно её: людей, которые проходят мимо входа, и машины, которые проезжают по аллее. Припаркованные машины не учитываем. Замеры в часы пик: утро 07:30–09:30, обед 12:30–14:30, вечер 17:30–20:00, отдельно выходные. По этим цифрам рассчитываем, сколько гостей и чеков реально получить в день. Результат: Отчёт с цифрами потока по часам и дням недели и расчётом ожидаемого числа чеков.</t>
+          <t xml:space="preserve">Поток у входа оценён расчётом: число квартир и жителей квартала, автомобили, способы передвижения и маршруты, которые проходят мимо входа. Получили поток по времени суток в будни и выходные и ожидаемое число чеков в день. Одночасовой контрольный счёт на месте утром буднего дня уточнит модель. Результат: Раздел отчёта «Локация, трафик и ожидаемый поток гостей»: поток по часам и дням недели, расчёт числа чеков с диапазоном.</t>
         </is>
       </c>
       <c r="N10" s="8"/>
@@ -1106,7 +1106,7 @@
         <f>G14-F14+1</f>
       </c>
       <c r="I14" s="6">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="J14" s="5" t="str">
         <f>IF(I14&gt;=1,"Готово",IF(G14&lt;TODAY(),"Просрочено",IF(F14&lt;=TODAY(),"В работе","В плане")))</f>

</xml_diff>

<commit_message>
Update plan 2026-10-10: traffic count
</commit_message>
<xml_diff>
--- a/pecan-plan.xlsx
+++ b/pecan-plan.xlsx
@@ -803,7 +803,7 @@
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Оценка трафика у входа: расчётная модель</t>
+          <t xml:space="preserve">Замер трафика у входа и оценка потока гостей</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
@@ -831,7 +831,7 @@
       <c r="L10" s="5"/>
       <c r="M10" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Поток у входа оценён расчётом: число квартир и жителей квартала, автомобили, способы передвижения и маршруты, которые проходят мимо входа. Получили поток по времени суток в будни и выходные и ожидаемое число чеков в день. Одночасовой контрольный счёт на месте утром буднего дня уточнит модель. Результат: Раздел отчёта «Локация, трафик и ожидаемый поток гостей»: поток по часам и дням недели, расчёт числа чеков с диапазоном.</t>
+          <t xml:space="preserve">Провели натурные замеры у входа 3–7 октября: пять сессий в будни и выходные, утро, обед и вечер. Считали пешеходов вдоль фасада и по аллее, автомобили на кольцевом проезде. Данные сверили с расчётной моделью квартала и получили ожидаемое число чеков в день. Результат: Отчёт по замеру трафика и раздел «Локация, трафик и ожидаемый поток гостей» в общем отчёте с анализом конкурентов: поток по дням и часам, расчёт числа чеков.</t>
         </is>
       </c>
       <c r="N10" s="8"/>

</xml_diff>